<commit_message>
Data update ma 18-05-2026
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -17238,7 +17238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2489"/>
+  <dimension ref="A1:I2590"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="20.140625" customWidth="1" min="1" max="1"/>
@@ -72723,6 +72723,3936 @@
         <v>46155</v>
       </c>
     </row>
+    <row r="2490">
+      <c r="A2490" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2490" t="n">
+        <v>5962</v>
+      </c>
+      <c r="C2490" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/queens-wilde-zalmfilet-met-huid</t>
+        </is>
+      </c>
+      <c r="D2490" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ZALMFILET MET HUID 375G</t>
+        </is>
+      </c>
+      <c r="E2490" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="F2490" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2490" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2490" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2490" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2491">
+      <c r="A2491" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2491" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2491" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/queens-pangalicious-knoflook-kruiden1</t>
+        </is>
+      </c>
+      <c r="D2491" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2491" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="F2491" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2491" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2491" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2491" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2492">
+      <c r="A2492" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2492" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2492" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/queens-pangalicious-ex-krokant</t>
+        </is>
+      </c>
+      <c r="D2492" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2492" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F2492" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2492" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2492" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2492" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2493">
+      <c r="A2493" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2493" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C2493" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/queens-pangalicious-citroen-peterselie1</t>
+        </is>
+      </c>
+      <c r="D2493" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS CITROEN &amp; PETERSELIE</t>
+        </is>
+      </c>
+      <c r="E2493" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="F2493" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2493" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2493" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2493" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2494">
+      <c r="A2494" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2494" t="n">
+        <v>27702</v>
+      </c>
+      <c r="C2494" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/the-ice-co-scherfijs</t>
+        </is>
+      </c>
+      <c r="D2494" t="inlineStr">
+        <is>
+          <t>528 CRUSHED ICE 1KG</t>
+        </is>
+      </c>
+      <c r="E2494" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="F2494" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2494" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2494" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2494" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2495">
+      <c r="A2495" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2495" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2495" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20pangalicious%20extra%20krokant/35468</t>
+        </is>
+      </c>
+      <c r="D2495" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2495" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F2495" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2495" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2495" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2495" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2496">
+      <c r="A2496" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2496" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2496" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20pangalicious%20knoflook%20kruiden/30297</t>
+        </is>
+      </c>
+      <c r="D2496" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2496" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="F2496" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2496" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2496" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2496" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2497">
+      <c r="A2497" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2497" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C2497" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307667</t>
+        </is>
+      </c>
+      <c r="D2497" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS CITROEN &amp; PETERSELIE</t>
+        </is>
+      </c>
+      <c r="E2497" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F2497" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2497" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2497" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2497" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2498">
+      <c r="A2498" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2498" t="n">
+        <v>5960</v>
+      </c>
+      <c r="C2498" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20pangafilet/42053</t>
+        </is>
+      </c>
+      <c r="D2498" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGAFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2498" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F2498" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2498" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2498" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2498" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2499">
+      <c r="A2499" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2499" t="n">
+        <v>5960</v>
+      </c>
+      <c r="C2499" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-panga-filets-375-g-419420ZK</t>
+        </is>
+      </c>
+      <c r="D2499" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGAFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2499" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F2499" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2499" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2499" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2499" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2500">
+      <c r="A2500" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2500" t="n">
+        <v>7001</v>
+      </c>
+      <c r="C2500" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-pangalicious-krokantjes-gekruid-pangasiusfilet-250g-697039DS</t>
+        </is>
+      </c>
+      <c r="D2500" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS VISKROKANTJES GEKRUID</t>
+        </is>
+      </c>
+      <c r="E2500" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2500" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2500" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2500" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2500" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2501">
+      <c r="A2501" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2501" t="n">
+        <v>5960</v>
+      </c>
+      <c r="C2501" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/queens-pangafilets2</t>
+        </is>
+      </c>
+      <c r="D2501" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGAFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2501" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F2501" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2501" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2501" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2501" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2502">
+      <c r="A2502" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2502" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C2502" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-pangalicious-krokantjes-naturel-pangasiusfilet-250-g-doos-697050DS</t>
+        </is>
+      </c>
+      <c r="D2502" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS VISKROKANTJES NATUREL</t>
+        </is>
+      </c>
+      <c r="E2502" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2502" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2502" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2502" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2502" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2503">
+      <c r="A2503" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2503" t="n">
+        <v>27208</v>
+      </c>
+      <c r="C2503" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/orienbites-gua-bao-320g-702769DS</t>
+        </is>
+      </c>
+      <c r="D2503" t="inlineStr">
+        <is>
+          <t>ORIEN BITES GUA BAO 320g</t>
+        </is>
+      </c>
+      <c r="E2503" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F2503" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2503" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2503" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2503" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2504">
+      <c r="A2504" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2504" t="n">
+        <v>6097</v>
+      </c>
+      <c r="C2504" t="inlineStr">
+        <is>
+          <t>https://www.aldi.nl/product-detail/gepaneerde-pangasiusfilets-1219976.html</t>
+        </is>
+      </c>
+      <c r="D2504" t="inlineStr">
+        <is>
+          <t>GOLDEN SEAFOOD ASC GEPANEERDE PANGASIUSFILET 6097</t>
+        </is>
+      </c>
+      <c r="E2504" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F2504" t="inlineStr">
+        <is>
+          <t>Aldi</t>
+        </is>
+      </c>
+      <c r="G2504" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2504" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2504" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2505">
+      <c r="A2505" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2505" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2505" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/queens-pangalicious-knoflook-kruiden-doos-250-g-439900</t>
+        </is>
+      </c>
+      <c r="D2505" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2505" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2505" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2505" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2505" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2505" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2506">
+      <c r="A2506" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2506" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C2506" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/queens-pangalicious-citroen-peterselie-doos-250-g-811995</t>
+        </is>
+      </c>
+      <c r="D2506" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS CITROEN &amp; PETERSELIE</t>
+        </is>
+      </c>
+      <c r="E2506" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2506" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2506" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2506" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2506" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2507">
+      <c r="A2507" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2507" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2507" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/queens-pangalicious-extra-krokant-doos-250-g-439896</t>
+        </is>
+      </c>
+      <c r="D2507" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2507" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F2507" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2507" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2507" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2507" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2508">
+      <c r="A2508" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2508" t="n">
+        <v>15594</v>
+      </c>
+      <c r="C2508" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/neutraal-knoflookbaguette-zak-175-g-455342</t>
+        </is>
+      </c>
+      <c r="D2508" t="inlineStr">
+        <is>
+          <t>KNOFLOOKBAGUETTE</t>
+        </is>
+      </c>
+      <c r="E2508" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F2508" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2508" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2508" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2508" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2509">
+      <c r="A2509" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2509" t="n">
+        <v>27701</v>
+      </c>
+      <c r="C2509" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/528-ijsblokjes-zak-2-kg-243144</t>
+        </is>
+      </c>
+      <c r="D2509" t="inlineStr">
+        <is>
+          <t>528 ICE CUBES 2KG</t>
+        </is>
+      </c>
+      <c r="E2509" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="F2509" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2509" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2509" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2509" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2510">
+      <c r="A2510" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2510" t="n">
+        <v>27703</v>
+      </c>
+      <c r="C2510" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/528-crushed-ice-zak-2-kg-318163</t>
+        </is>
+      </c>
+      <c r="D2510" t="inlineStr">
+        <is>
+          <t>528 CRUSHED ICE 2KG</t>
+        </is>
+      </c>
+      <c r="E2510" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="F2510" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2510" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2510" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2510" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2511">
+      <c r="A2511" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2511" t="n">
+        <v>5961</v>
+      </c>
+      <c r="C2511" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-alaska-koolvis-filets-375-g-419422ZK</t>
+        </is>
+      </c>
+      <c r="D2511" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ALASKA KOOLVISFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2511" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="F2511" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2511" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2511" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2511" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2512">
+      <c r="A2512" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2512" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2512" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/queens-panga-extra-krokant/148518</t>
+        </is>
+      </c>
+      <c r="D2512" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2512" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F2512" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2512" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2512" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2512" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2513">
+      <c r="A2513" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2513" t="n">
+        <v>27704</v>
+      </c>
+      <c r="C2513" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/528-ijsballen-1-kg-741532ZK</t>
+        </is>
+      </c>
+      <c r="D2513" t="inlineStr">
+        <is>
+          <t>528 ICE BALLS 1KG</t>
+        </is>
+      </c>
+      <c r="E2513" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="F2513" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2513" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2513" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2513" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2514">
+      <c r="A2514" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2514" t="n">
+        <v>5962</v>
+      </c>
+      <c r="C2514" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20wilde%20zalmfilets%20met%20huid/59292</t>
+        </is>
+      </c>
+      <c r="D2514" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ZALMFILET MET HUID 375G</t>
+        </is>
+      </c>
+      <c r="E2514" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="F2514" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2514" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2514" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2514" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2515">
+      <c r="A2515" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2515" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2515" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-pangalicious-extra-krokant-2-stuks-250-g-184995DS</t>
+        </is>
+      </c>
+      <c r="D2515" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2515" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F2515" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2515" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2515" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2515" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2516">
+      <c r="A2516" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2516" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2516" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-pangalicious-knoflook-kruiden-2-stuks-250-g-184996DS</t>
+        </is>
+      </c>
+      <c r="D2516" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2516" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2516" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2516" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2516" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2516" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2517">
+      <c r="A2517" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2517" t="n">
+        <v>6989</v>
+      </c>
+      <c r="C2517" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi212118/ah-ijsblokjes</t>
+        </is>
+      </c>
+      <c r="D2517" t="inlineStr">
+        <is>
+          <t>ALBERT HEIJN IJSBLOKJES 1KG</t>
+        </is>
+      </c>
+      <c r="E2517" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F2517" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2517" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2517" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2517" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2518">
+      <c r="A2518" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2518" t="n">
+        <v>27704</v>
+      </c>
+      <c r="C2518" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi589548/528-premium-ice-balls</t>
+        </is>
+      </c>
+      <c r="D2518" t="inlineStr">
+        <is>
+          <t>528 ICE BALLS 1KG</t>
+        </is>
+      </c>
+      <c r="E2518" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="F2518" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2518" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2518" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2518" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2519">
+      <c r="A2519" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2519" t="n">
+        <v>6541</v>
+      </c>
+      <c r="C2519" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-pangalicious-pikant-gekruid-2-stuks-250-g-550475DS</t>
+        </is>
+      </c>
+      <c r="D2519" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS PIKANT GEKRUID</t>
+        </is>
+      </c>
+      <c r="E2519" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="F2519" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2519" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2519" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2519" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2520">
+      <c r="A2520" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2520" t="n">
+        <v>6673</v>
+      </c>
+      <c r="C2520" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-kabeljauwfilet-met-huid-375g-705923ZK</t>
+        </is>
+      </c>
+      <c r="D2520" t="inlineStr">
+        <is>
+          <t>QUEENS MSC KABELJAUWFILETS MET HUID 375G</t>
+        </is>
+      </c>
+      <c r="E2520" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="F2520" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2520" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2520" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2520" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2521">
+      <c r="A2521" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2521" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C2521" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-pangalicious-citroen-peterselie-2-stuks-250-g-184997DS</t>
+        </is>
+      </c>
+      <c r="D2521" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS CITROEN &amp; PETERSELIE</t>
+        </is>
+      </c>
+      <c r="E2521" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2521" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2521" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2521" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2521" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2522">
+      <c r="A2522" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2522" t="n">
+        <v>27702</v>
+      </c>
+      <c r="C2522" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/ijs/crushed%20ijs/116221</t>
+        </is>
+      </c>
+      <c r="D2522" t="inlineStr">
+        <is>
+          <t>528 CRUSHED ICE 1KG</t>
+        </is>
+      </c>
+      <c r="E2522" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F2522" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2522" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2522" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2522" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2523">
+      <c r="A2523" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2523" t="n">
+        <v>5961</v>
+      </c>
+      <c r="C2523" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20alaska%20koolvisfilet/42054</t>
+        </is>
+      </c>
+      <c r="D2523" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ALASKA KOOLVISFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2523" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2523" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2523" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2523" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2523" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2524">
+      <c r="A2524" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2524" t="n">
+        <v>15594</v>
+      </c>
+      <c r="C2524" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-snacks/queens%20baguette%20met%20knoflookboter/118061</t>
+        </is>
+      </c>
+      <c r="D2524" t="inlineStr">
+        <is>
+          <t>KNOFLOOKBAGUETTE</t>
+        </is>
+      </c>
+      <c r="F2524" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2524" t="inlineStr">
+        <is>
+          <t>Geen prijs gevonden</t>
+        </is>
+      </c>
+      <c r="H2524" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2524" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2525">
+      <c r="A2525" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2525" t="n">
+        <v>5962</v>
+      </c>
+      <c r="C2525" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/queens-wilde-zalmfilet/154077</t>
+        </is>
+      </c>
+      <c r="D2525" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ZALMFILET MET HUID 375G</t>
+        </is>
+      </c>
+      <c r="E2525" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="F2525" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2525" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2525" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2525" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2526">
+      <c r="A2526" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2526" t="n">
+        <v>27702</v>
+      </c>
+      <c r="C2526" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/ijs/crushed%20ijs/116221</t>
+        </is>
+      </c>
+      <c r="D2526" t="inlineStr">
+        <is>
+          <t>528 CRUSHED ICE 1KG</t>
+        </is>
+      </c>
+      <c r="F2526" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2526" t="inlineStr">
+        <is>
+          <t>Geen prijs gevonden</t>
+        </is>
+      </c>
+      <c r="H2526" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2526" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2527">
+      <c r="A2527" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2527" t="n">
+        <v>5962</v>
+      </c>
+      <c r="C2527" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20wilde%20zalmfilets%20met%20huid/59292</t>
+        </is>
+      </c>
+      <c r="D2527" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ZALMFILET MET HUID 375G</t>
+        </is>
+      </c>
+      <c r="E2527" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="F2527" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2527" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2527" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2527" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2528">
+      <c r="A2528" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2528" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2528" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20pangalicious%20knoflook%20kruiden/30297</t>
+        </is>
+      </c>
+      <c r="D2528" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2528" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="F2528" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2528" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2528" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2528" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2529">
+      <c r="A2529" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2529" t="n">
+        <v>5961</v>
+      </c>
+      <c r="C2529" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20alaska%20koolvisfilet/42054</t>
+        </is>
+      </c>
+      <c r="D2529" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ALASKA KOOLVISFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2529" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="F2529" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2529" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2529" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2529" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2530">
+      <c r="A2530" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2530" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C2530" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20pangalicious%20citroen-peterselie/32212</t>
+        </is>
+      </c>
+      <c r="D2530" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS CITROEN &amp; PETERSELIE</t>
+        </is>
+      </c>
+      <c r="E2530" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="F2530" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2530" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2530" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2530" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2531">
+      <c r="A2531" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2531" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2531" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20pangalicious%20extra%20krokant/35468</t>
+        </is>
+      </c>
+      <c r="D2531" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2531" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="F2531" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2531" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2531" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2531" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2532">
+      <c r="A2532" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2532" t="n">
+        <v>6541</v>
+      </c>
+      <c r="C2532" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20pangasiusfilet%20pikant%20gekruid/87324</t>
+        </is>
+      </c>
+      <c r="D2532" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS PIKANT GEKRUID</t>
+        </is>
+      </c>
+      <c r="E2532" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="F2532" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2532" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2532" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2532" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2533">
+      <c r="A2533" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2533" t="n">
+        <v>5960</v>
+      </c>
+      <c r="C2533" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/queens-pangafilets-375gr/134358</t>
+        </is>
+      </c>
+      <c r="D2533" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGAFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2533" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F2533" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2533" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2533" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2533" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2534">
+      <c r="A2534" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2534" t="n">
+        <v>6673</v>
+      </c>
+      <c r="C2534" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20kabeljauwfilet%20met%20huid/115384</t>
+        </is>
+      </c>
+      <c r="D2534" t="inlineStr">
+        <is>
+          <t>QUEENS MSC KABELJAUWFILETS MET HUID 375G</t>
+        </is>
+      </c>
+      <c r="E2534" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="F2534" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2534" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2534" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2534" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2535">
+      <c r="A2535" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2535" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2535" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/queens-panga-knof-kruid-250gr/125556</t>
+        </is>
+      </c>
+      <c r="D2535" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2535" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="F2535" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2535" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2535" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2535" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2536">
+      <c r="A2536" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2536" t="n">
+        <v>5961</v>
+      </c>
+      <c r="C2536" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/queens-koolvis-375gr/137392</t>
+        </is>
+      </c>
+      <c r="D2536" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ALASKA KOOLVISFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2536" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2536" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2536" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2536" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2536" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2537">
+      <c r="A2537" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2537" t="n">
+        <v>5960</v>
+      </c>
+      <c r="C2537" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20pangafilet/42053</t>
+        </is>
+      </c>
+      <c r="D2537" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGAFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2537" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="F2537" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2537" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2537" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2537" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2538">
+      <c r="A2538" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2538" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2538" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307666</t>
+        </is>
+      </c>
+      <c r="D2538" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2538" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F2538" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2538" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2538" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2538" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2539">
+      <c r="A2539" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2539" t="n">
+        <v/>
+      </c>
+      <c r="C2539" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/vis-marine-wilde-zalm</t>
+        </is>
+      </c>
+      <c r="D2539" t="inlineStr">
+        <is>
+          <t>Vis Marine Wilde zalm 540g</t>
+        </is>
+      </c>
+      <c r="E2539" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="F2539" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2539" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2539" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2539" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2540">
+      <c r="A2540" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2540" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2540" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307674</t>
+        </is>
+      </c>
+      <c r="D2540" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2540" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F2540" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2540" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2540" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2540" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2541">
+      <c r="A2541" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2541" t="n">
+        <v/>
+      </c>
+      <c r="C2541" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/vis-marine-kabeljauwfilets</t>
+        </is>
+      </c>
+      <c r="D2541" t="inlineStr">
+        <is>
+          <t>Vis Marine Kabeljauw 400g</t>
+        </is>
+      </c>
+      <c r="E2541" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="F2541" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2541" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2541" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2541" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2542">
+      <c r="A2542" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2542" t="n">
+        <v>27207</v>
+      </c>
+      <c r="C2542" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307850</t>
+        </is>
+      </c>
+      <c r="D2542" t="inlineStr">
+        <is>
+          <t>ORIEN BITES CHICKEN GYOZA</t>
+        </is>
+      </c>
+      <c r="E2542" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="F2542" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2542" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2542" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2542" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2543">
+      <c r="A2543" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2543" t="n">
+        <v>27200</v>
+      </c>
+      <c r="C2543" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307851</t>
+        </is>
+      </c>
+      <c r="D2543" t="inlineStr">
+        <is>
+          <t>ORIEN BITES VEG GYOZA</t>
+        </is>
+      </c>
+      <c r="E2543" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="F2543" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2543" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2543" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2543" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2544">
+      <c r="A2544" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2544" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2544" t="inlineStr">
+        <is>
+          <t>https://www.spar.nl/queens-pangafilet-knoflook-kruiden-1998285/</t>
+        </is>
+      </c>
+      <c r="D2544" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2544" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="F2544" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="G2544" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2544" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2544" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2545">
+      <c r="A2545" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2545" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C2545" t="inlineStr">
+        <is>
+          <t>https://www.spar.nl/queens-pangasius-filet-citroen-peterselie-2730456/</t>
+        </is>
+      </c>
+      <c r="D2545" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS CITROEN &amp; PETERSELIE</t>
+        </is>
+      </c>
+      <c r="E2545" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="F2545" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="G2545" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2545" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2545" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2546">
+      <c r="A2546" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2546" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2546" t="inlineStr">
+        <is>
+          <t>https://www.spar.nl/queens-pangalicious-9158971/</t>
+        </is>
+      </c>
+      <c r="D2546" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2546" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="F2546" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="G2546" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2546" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2546" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2547">
+      <c r="A2547" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2547" t="n">
+        <v/>
+      </c>
+      <c r="C2547" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/vis%20marine%20koolvisfilet%204%20stuks/49562</t>
+        </is>
+      </c>
+      <c r="D2547" t="inlineStr">
+        <is>
+          <t>Vis Marine Koolvis 400g</t>
+        </is>
+      </c>
+      <c r="E2547" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F2547" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2547" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2547" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2547" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2548">
+      <c r="A2548" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2548" t="n">
+        <v/>
+      </c>
+      <c r="C2548" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/vis%20marine%20kabeljauwfilet%204%20stuks/49672</t>
+        </is>
+      </c>
+      <c r="D2548" t="inlineStr">
+        <is>
+          <t>Vis Marine Kabeljauw 400g</t>
+        </is>
+      </c>
+      <c r="E2548" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="F2548" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2548" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2548" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2548" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2549">
+      <c r="A2549" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2549" t="n">
+        <v/>
+      </c>
+      <c r="C2549" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/vis%20marine%20pangasiusfilet/82503</t>
+        </is>
+      </c>
+      <c r="D2549" t="inlineStr">
+        <is>
+          <t>Vis Marine Pangasiusfilet 540g</t>
+        </is>
+      </c>
+      <c r="E2549" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="F2549" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2549" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2549" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2549" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2550">
+      <c r="A2550" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2550" t="n">
+        <v/>
+      </c>
+      <c r="C2550" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/vis%20marine%20wilde%20zalm/96927</t>
+        </is>
+      </c>
+      <c r="D2550" t="inlineStr">
+        <is>
+          <t>Vis Marine Wilde zalm 540g</t>
+        </is>
+      </c>
+      <c r="E2550" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="F2550" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2550" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2550" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2550" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2551">
+      <c r="A2551" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2551" t="n">
+        <v/>
+      </c>
+      <c r="C2551" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/vis-marine-koolvisfilets-doos-400-g-834796</t>
+        </is>
+      </c>
+      <c r="D2551" t="inlineStr">
+        <is>
+          <t>Vis Marine Koolvis 400g</t>
+        </is>
+      </c>
+      <c r="E2551" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F2551" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2551" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2551" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2551" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2552">
+      <c r="A2552" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2552" t="n">
+        <v>27700</v>
+      </c>
+      <c r="C2552" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/309633</t>
+        </is>
+      </c>
+      <c r="D2552" t="inlineStr">
+        <is>
+          <t>528 ICE CUBES 1KG</t>
+        </is>
+      </c>
+      <c r="E2552" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F2552" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2552" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2552" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2552" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2553">
+      <c r="A2553" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2553" t="n">
+        <v/>
+      </c>
+      <c r="C2553" t="inlineStr">
+        <is>
+          <t>https://www.spar.nl/vis-marine-kabeljauwfilets-4-stuks-9228133/</t>
+        </is>
+      </c>
+      <c r="D2553" t="inlineStr">
+        <is>
+          <t>Vis Marine Kabeljauw 400g</t>
+        </is>
+      </c>
+      <c r="E2553" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F2553" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="G2553" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2553" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2553" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2554">
+      <c r="A2554" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2554" t="n">
+        <v/>
+      </c>
+      <c r="C2554" t="inlineStr">
+        <is>
+          <t>https://www.spar.nl/vis-marine-pangasius-filets-9188805/</t>
+        </is>
+      </c>
+      <c r="D2554" t="inlineStr">
+        <is>
+          <t>Vis Marine Pangasiusfilet 540g</t>
+        </is>
+      </c>
+      <c r="E2554" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F2554" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="G2554" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2554" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2554" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2555">
+      <c r="A2555" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2555" t="n">
+        <v/>
+      </c>
+      <c r="C2555" t="inlineStr">
+        <is>
+          <t>https://www.spar.nl/vis-marine-wilde-zalmfilet-9194254/</t>
+        </is>
+      </c>
+      <c r="D2555" t="inlineStr">
+        <is>
+          <t>Vis Marine Wilde zalm 540g</t>
+        </is>
+      </c>
+      <c r="E2555" t="n">
+        <v>6.59</v>
+      </c>
+      <c r="F2555" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="G2555" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2555" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2555" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2556">
+      <c r="A2556" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2556" t="n">
+        <v/>
+      </c>
+      <c r="C2556" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307411</t>
+        </is>
+      </c>
+      <c r="D2556" t="inlineStr">
+        <is>
+          <t>Vis Marine Koolvis 400g</t>
+        </is>
+      </c>
+      <c r="E2556" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="F2556" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2556" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2556" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2556" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2557">
+      <c r="A2557" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2557" t="n">
+        <v/>
+      </c>
+      <c r="C2557" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307028</t>
+        </is>
+      </c>
+      <c r="D2557" t="inlineStr">
+        <is>
+          <t>Vis Marine Kabeljauw 540g</t>
+        </is>
+      </c>
+      <c r="E2557" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="F2557" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2557" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2557" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2557" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2558">
+      <c r="A2558" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2558" t="n">
+        <v/>
+      </c>
+      <c r="C2558" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307026</t>
+        </is>
+      </c>
+      <c r="D2558" t="inlineStr">
+        <is>
+          <t>Vis Marine Pangasiusfilet 540g</t>
+        </is>
+      </c>
+      <c r="E2558" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="F2558" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2558" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2558" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2558" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2559">
+      <c r="A2559" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2559" t="n">
+        <v/>
+      </c>
+      <c r="C2559" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307023</t>
+        </is>
+      </c>
+      <c r="D2559" t="inlineStr">
+        <is>
+          <t>Vis Marine Wilde zalm 540g</t>
+        </is>
+      </c>
+      <c r="E2559" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F2559" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2559" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2559" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2559" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2560">
+      <c r="A2560" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2560" t="n">
+        <v/>
+      </c>
+      <c r="C2560" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/vis-marine-koolvisfilets</t>
+        </is>
+      </c>
+      <c r="D2560" t="inlineStr">
+        <is>
+          <t>Vis Marine Koolvis 400g</t>
+        </is>
+      </c>
+      <c r="E2560" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F2560" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2560" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2560" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2560" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2561">
+      <c r="A2561" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2561" t="n">
+        <v/>
+      </c>
+      <c r="C2561" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/plus-tilapiafilets-zak-540-g-793166?utm_source=awin&amp;utm_medium=affiliate&amp;utm_campaign=531573_ShopForward+CSS&amp;utm_content=0&amp;sv1=affiliate&amp;sv_campaign_id=531573&amp;awc=12479_1776164499_4fdb47ad85457250f177963ef4cdf5d9</t>
+        </is>
+      </c>
+      <c r="D2561" t="inlineStr">
+        <is>
+          <t>Plus Tilapiafilets 540g</t>
+        </is>
+      </c>
+      <c r="E2561" t="n">
+        <v>496.45</v>
+      </c>
+      <c r="F2561" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2561" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2561" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2561" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2562">
+      <c r="A2562" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2562" t="n">
+        <v>27704</v>
+      </c>
+      <c r="C2562" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/528-ijsballen-zak-1-kg-769217</t>
+        </is>
+      </c>
+      <c r="D2562" t="inlineStr">
+        <is>
+          <t>528 ICE BALLS 1KG</t>
+        </is>
+      </c>
+      <c r="E2562" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="F2562" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2562" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2562" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2562" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2563">
+      <c r="A2563" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2563" t="n">
+        <v/>
+      </c>
+      <c r="C2563" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/vis-marine-kabeljauwfilets-msc-doos-540-g-723219</t>
+        </is>
+      </c>
+      <c r="D2563" t="inlineStr">
+        <is>
+          <t>Vis Marine Kabeljauw 540g</t>
+        </is>
+      </c>
+      <c r="E2563" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="F2563" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2563" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2563" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2563" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2564">
+      <c r="A2564" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2564" t="n">
+        <v>6541</v>
+      </c>
+      <c r="C2564" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20pangasiusfilet%20pikant%20gekruid/87324</t>
+        </is>
+      </c>
+      <c r="D2564" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS PIKANT GEKRUID</t>
+        </is>
+      </c>
+      <c r="E2564" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F2564" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2564" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2564" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2564" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2565">
+      <c r="A2565" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2565" t="n">
+        <v/>
+      </c>
+      <c r="C2565" t="inlineStr">
+        <is>
+          <t>https://www.aldi.nl/product/wilde-zalmfilets-1204877.html</t>
+        </is>
+      </c>
+      <c r="D2565" t="inlineStr">
+        <is>
+          <t>Aldi Wilde zalmfilet 500g</t>
+        </is>
+      </c>
+      <c r="E2565" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="F2565" t="inlineStr">
+        <is>
+          <t>Aldi</t>
+        </is>
+      </c>
+      <c r="G2565" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2565" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2565" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2566">
+      <c r="A2566" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2566" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C2566" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307713</t>
+        </is>
+      </c>
+      <c r="D2566" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS VISKROKANTJES NATUREL</t>
+        </is>
+      </c>
+      <c r="E2566" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F2566" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2566" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2566" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2566" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2567">
+      <c r="A2567" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2567" t="n">
+        <v/>
+      </c>
+      <c r="C2567" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-zalmfilet-met-huid-2-x-125-g-723226DS</t>
+        </is>
+      </c>
+      <c r="D2567" t="inlineStr">
+        <is>
+          <t>Jumbo Zalmfilet met Huid 2 x 125g</t>
+        </is>
+      </c>
+      <c r="E2567" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="F2567" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2567" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2567" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2567" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2568">
+      <c r="A2568" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2568" t="n">
+        <v/>
+      </c>
+      <c r="C2568" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis%20marine%20koolvisfilet%204%20stuks/49562</t>
+        </is>
+      </c>
+      <c r="D2568" t="inlineStr">
+        <is>
+          <t>Vis Marine Koolvis 400g</t>
+        </is>
+      </c>
+      <c r="E2568" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F2568" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2568" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2568" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2568" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2569">
+      <c r="A2569" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2569" t="n">
+        <v/>
+      </c>
+      <c r="C2569" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis%20marine%20kabeljauwfilets/111544</t>
+        </is>
+      </c>
+      <c r="D2569" t="inlineStr">
+        <is>
+          <t>Vis Marine Kabeljauw 540g</t>
+        </is>
+      </c>
+      <c r="F2569" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2569" t="inlineStr">
+        <is>
+          <t>Niet beschikbaar</t>
+        </is>
+      </c>
+      <c r="H2569" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2569" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2570">
+      <c r="A2570" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2570" t="n">
+        <v/>
+      </c>
+      <c r="C2570" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis%20marine%20pangasiusfilet/82503</t>
+        </is>
+      </c>
+      <c r="D2570" t="inlineStr">
+        <is>
+          <t>Vis Marine Pangasiusfilet 540g</t>
+        </is>
+      </c>
+      <c r="E2570" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="F2570" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2570" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2570" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2570" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2571">
+      <c r="A2571" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2571" t="n">
+        <v/>
+      </c>
+      <c r="C2571" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis%20marine%20wilde%20zalm/96927</t>
+        </is>
+      </c>
+      <c r="D2571" t="inlineStr">
+        <is>
+          <t>Vis Marine Wilde zalm 540g</t>
+        </is>
+      </c>
+      <c r="E2571" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="F2571" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2571" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2571" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2571" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2572">
+      <c r="A2572" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2572" t="n">
+        <v/>
+      </c>
+      <c r="C2572" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis-marine-tilapia-filets-5-6-st/83124</t>
+        </is>
+      </c>
+      <c r="D2572" t="inlineStr">
+        <is>
+          <t>Vis Marine Tilapiafilets 540g</t>
+        </is>
+      </c>
+      <c r="E2572" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="F2572" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2572" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2572" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2572" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2573">
+      <c r="A2573" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2573" t="n">
+        <v/>
+      </c>
+      <c r="C2573" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-koolvis-filet-400-g-713748DS</t>
+        </is>
+      </c>
+      <c r="D2573" t="inlineStr">
+        <is>
+          <t>Jumbo Koolvis Filet 400g</t>
+        </is>
+      </c>
+      <c r="E2573" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F2573" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2573" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2573" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2573" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2574">
+      <c r="A2574" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2574" t="n">
+        <v/>
+      </c>
+      <c r="C2574" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/seacon-alaska-koolvisfilet-675g-706749ZK</t>
+        </is>
+      </c>
+      <c r="D2574" t="inlineStr">
+        <is>
+          <t>Seacon Alaska Koolvisfilet 675g</t>
+        </is>
+      </c>
+      <c r="E2574" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="F2574" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2574" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2574" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2574" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2575">
+      <c r="A2575" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2575" t="n">
+        <v/>
+      </c>
+      <c r="C2575" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-kabeljauwfilet-675-g-471158ZK</t>
+        </is>
+      </c>
+      <c r="D2575" t="inlineStr">
+        <is>
+          <t>Jumbo Kabeljauwfilet 675g</t>
+        </is>
+      </c>
+      <c r="E2575" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="F2575" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2575" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2575" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2575" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2576">
+      <c r="A2576" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2576" t="n">
+        <v/>
+      </c>
+      <c r="C2576" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-pangasiusfilet-vriesvers-675-g-494433ZK</t>
+        </is>
+      </c>
+      <c r="D2576" t="inlineStr">
+        <is>
+          <t>Jumbo Pangasiusfilet Vriesvers 675g</t>
+        </is>
+      </c>
+      <c r="E2576" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="F2576" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2576" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2576" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2576" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2577">
+      <c r="A2577" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2577" t="n">
+        <v/>
+      </c>
+      <c r="C2577" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/vismarine-pangasiusfilet-540gr/110960</t>
+        </is>
+      </c>
+      <c r="D2577" t="inlineStr">
+        <is>
+          <t>Vis Marine Pangasiusfilet 540g</t>
+        </is>
+      </c>
+      <c r="E2577" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="F2577" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2577" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2577" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2577" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2578">
+      <c r="A2578" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2578" t="n">
+        <v/>
+      </c>
+      <c r="C2578" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-pangasiusfilet-270-g-173837ZK</t>
+        </is>
+      </c>
+      <c r="D2578" t="inlineStr">
+        <is>
+          <t>Jumbo Pangasiusfilet 270g</t>
+        </is>
+      </c>
+      <c r="E2578" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="F2578" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2578" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2578" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2578" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2579">
+      <c r="A2579" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2579" t="n">
+        <v/>
+      </c>
+      <c r="C2579" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/vismarine-koolvisfilet-4stmsc/811408</t>
+        </is>
+      </c>
+      <c r="D2579" t="inlineStr">
+        <is>
+          <t>Vis Marine Koolvis 400g</t>
+        </is>
+      </c>
+      <c r="E2579" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F2579" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2579" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2579" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2579" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2580">
+      <c r="A2580" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2580" t="n">
+        <v/>
+      </c>
+      <c r="C2580" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-wilde-zalmfilet-2-x-125-g-76159PAK</t>
+        </is>
+      </c>
+      <c r="D2580" t="inlineStr">
+        <is>
+          <t>Jumbo Wilde Zalmfilet 2 x 125g</t>
+        </is>
+      </c>
+      <c r="E2580" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="F2580" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2580" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2580" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2580" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2581">
+      <c r="A2581" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2581" t="n">
+        <v/>
+      </c>
+      <c r="C2581" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi39826/ah-koolvisfilet</t>
+        </is>
+      </c>
+      <c r="D2581" t="inlineStr">
+        <is>
+          <t>AH Koolvisfilet 400g</t>
+        </is>
+      </c>
+      <c r="E2581" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="F2581" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2581" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2581" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2581" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2582">
+      <c r="A2582" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2582" t="n">
+        <v/>
+      </c>
+      <c r="C2582" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi121478/ah-kabeljauwfilet</t>
+        </is>
+      </c>
+      <c r="D2582" t="inlineStr">
+        <is>
+          <t>AH Kabeljauwfilet 675g</t>
+        </is>
+      </c>
+      <c r="E2582" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="F2582" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2582" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2582" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2582" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2583">
+      <c r="A2583" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2583" t="n">
+        <v/>
+      </c>
+      <c r="C2583" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi792/ah-kabeljauw</t>
+        </is>
+      </c>
+      <c r="D2583" t="inlineStr">
+        <is>
+          <t>AH Kabeljauw 400g</t>
+        </is>
+      </c>
+      <c r="E2583" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="F2583" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2583" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2583" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2583" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2584">
+      <c r="A2584" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2584" t="n">
+        <v/>
+      </c>
+      <c r="C2584" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi140671/ah-pangasiusfilet</t>
+        </is>
+      </c>
+      <c r="D2584" t="inlineStr">
+        <is>
+          <t>AH Pangasiusfilet 675g</t>
+        </is>
+      </c>
+      <c r="E2584" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="F2584" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2584" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2584" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2584" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2585">
+      <c r="A2585" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2585" t="n">
+        <v/>
+      </c>
+      <c r="C2585" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi141565/ah-wilde-zalmfilets</t>
+        </is>
+      </c>
+      <c r="D2585" t="inlineStr">
+        <is>
+          <t>AH Wilde zalmfilet 675g</t>
+        </is>
+      </c>
+      <c r="E2585" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="F2585" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2585" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2585" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2585" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2586">
+      <c r="A2586" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2586" t="n">
+        <v/>
+      </c>
+      <c r="C2586" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi178129/ah-wilde-zalmfilet</t>
+        </is>
+      </c>
+      <c r="D2586" t="inlineStr">
+        <is>
+          <t>AH Wilde zalmfilet 250g</t>
+        </is>
+      </c>
+      <c r="E2586" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="F2586" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2586" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2586" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2586" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2587">
+      <c r="A2587" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2587" t="n">
+        <v/>
+      </c>
+      <c r="C2587" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi396815/ah-tilapiafilet-graatvrij</t>
+        </is>
+      </c>
+      <c r="D2587" t="inlineStr">
+        <is>
+          <t>AH Tilapiafilet graatvrij 225g</t>
+        </is>
+      </c>
+      <c r="E2587" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F2587" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2587" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2587" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2587" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2588">
+      <c r="A2588" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2588" t="n">
+        <v/>
+      </c>
+      <c r="C2588" t="inlineStr">
+        <is>
+          <t>https://www.aldi.nl/product/pangasiusfilet-1221684.html</t>
+        </is>
+      </c>
+      <c r="D2588" t="inlineStr">
+        <is>
+          <t>Aldi Pangasiusfilet 540g</t>
+        </is>
+      </c>
+      <c r="E2588" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="F2588" t="inlineStr">
+        <is>
+          <t>Aldi</t>
+        </is>
+      </c>
+      <c r="G2588" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2588" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2588" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2589">
+      <c r="A2589" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2589" t="n">
+        <v/>
+      </c>
+      <c r="C2589" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-wilde-zalm-filet-675-g-487780ZK</t>
+        </is>
+      </c>
+      <c r="D2589" t="inlineStr">
+        <is>
+          <t>Jumbo Wilde Zalm Filet 675g</t>
+        </is>
+      </c>
+      <c r="E2589" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F2589" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2589" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2589" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2589" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2590">
+      <c r="A2590" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2590" t="n">
+        <v>27300</v>
+      </c>
+      <c r="C2590" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-brood-bladerdeeg/knoflookbaguette-175gr/301172</t>
+        </is>
+      </c>
+      <c r="D2590" t="inlineStr">
+        <is>
+          <t>KNOFLOOKBAGUETTE</t>
+        </is>
+      </c>
+      <c r="E2590" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="F2590" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2590" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2590" s="13" t="n">
+        <v>46160</v>
+      </c>
+      <c r="I2590" t="n">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId1"/>

</xml_diff>

<commit_message>
Foutieve prijs Plus Tilapia gecorrigeerd (496.45 -> 6.45)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -71847,6 +71847,306 @@
     <row r="1562" ht="15" customHeight="1">
       <c r="H1562" s="1" t="n"/>
     </row>
+    <row r="1563"/>
+    <row r="1564"/>
+    <row r="1565"/>
+    <row r="1566"/>
+    <row r="1567"/>
+    <row r="1568"/>
+    <row r="1569"/>
+    <row r="1570"/>
+    <row r="1571"/>
+    <row r="1572"/>
+    <row r="1573"/>
+    <row r="1574"/>
+    <row r="1575"/>
+    <row r="1576"/>
+    <row r="1577"/>
+    <row r="1578"/>
+    <row r="1579"/>
+    <row r="1580"/>
+    <row r="1581"/>
+    <row r="1582"/>
+    <row r="1583"/>
+    <row r="1584"/>
+    <row r="1585"/>
+    <row r="1586"/>
+    <row r="1587"/>
+    <row r="1588"/>
+    <row r="1589"/>
+    <row r="1590"/>
+    <row r="1591"/>
+    <row r="1592"/>
+    <row r="1593"/>
+    <row r="1594"/>
+    <row r="1595"/>
+    <row r="1596"/>
+    <row r="1597"/>
+    <row r="1598"/>
+    <row r="1599"/>
+    <row r="1600"/>
+    <row r="1601"/>
+    <row r="1602"/>
+    <row r="1603"/>
+    <row r="1604"/>
+    <row r="1605"/>
+    <row r="1606"/>
+    <row r="1607"/>
+    <row r="1608"/>
+    <row r="1609"/>
+    <row r="1610"/>
+    <row r="1611"/>
+    <row r="1612"/>
+    <row r="1613"/>
+    <row r="1614"/>
+    <row r="1615"/>
+    <row r="1616"/>
+    <row r="1617"/>
+    <row r="1618"/>
+    <row r="1619"/>
+    <row r="1620"/>
+    <row r="1621"/>
+    <row r="1622"/>
+    <row r="1623"/>
+    <row r="1624"/>
+    <row r="1625"/>
+    <row r="1626"/>
+    <row r="1627"/>
+    <row r="1628"/>
+    <row r="1629"/>
+    <row r="1630"/>
+    <row r="1631"/>
+    <row r="1632"/>
+    <row r="1633"/>
+    <row r="1634"/>
+    <row r="1635"/>
+    <row r="1636"/>
+    <row r="1637"/>
+    <row r="1638"/>
+    <row r="1639"/>
+    <row r="1640"/>
+    <row r="1641"/>
+    <row r="1642"/>
+    <row r="1643"/>
+    <row r="1644"/>
+    <row r="1645"/>
+    <row r="1646"/>
+    <row r="1647"/>
+    <row r="1648"/>
+    <row r="1649"/>
+    <row r="1650"/>
+    <row r="1651"/>
+    <row r="1652"/>
+    <row r="1653"/>
+    <row r="1654"/>
+    <row r="1655"/>
+    <row r="1656"/>
+    <row r="1657"/>
+    <row r="1658"/>
+    <row r="1659"/>
+    <row r="1660"/>
+    <row r="1661"/>
+    <row r="1662"/>
+    <row r="1663"/>
+    <row r="1664"/>
+    <row r="1665"/>
+    <row r="1666"/>
+    <row r="1667"/>
+    <row r="1668"/>
+    <row r="1669"/>
+    <row r="1670"/>
+    <row r="1671"/>
+    <row r="1672"/>
+    <row r="1673"/>
+    <row r="1674"/>
+    <row r="1675"/>
+    <row r="1676"/>
+    <row r="1677"/>
+    <row r="1678"/>
+    <row r="1679"/>
+    <row r="1680"/>
+    <row r="1681"/>
+    <row r="1682"/>
+    <row r="1683"/>
+    <row r="1684"/>
+    <row r="1685"/>
+    <row r="1686"/>
+    <row r="1687"/>
+    <row r="1688"/>
+    <row r="1689"/>
+    <row r="1690"/>
+    <row r="1691"/>
+    <row r="1692"/>
+    <row r="1693"/>
+    <row r="1694"/>
+    <row r="1695"/>
+    <row r="1696"/>
+    <row r="1697"/>
+    <row r="1698"/>
+    <row r="1699"/>
+    <row r="1700"/>
+    <row r="1701"/>
+    <row r="1702"/>
+    <row r="1703"/>
+    <row r="1704"/>
+    <row r="1705"/>
+    <row r="1706"/>
+    <row r="1707"/>
+    <row r="1708"/>
+    <row r="1709"/>
+    <row r="1710"/>
+    <row r="1711"/>
+    <row r="1712"/>
+    <row r="1713"/>
+    <row r="1714"/>
+    <row r="1715"/>
+    <row r="1716"/>
+    <row r="1717"/>
+    <row r="1718"/>
+    <row r="1719"/>
+    <row r="1720"/>
+    <row r="1721"/>
+    <row r="1722"/>
+    <row r="1723"/>
+    <row r="1724"/>
+    <row r="1725"/>
+    <row r="1726"/>
+    <row r="1727"/>
+    <row r="1728"/>
+    <row r="1729"/>
+    <row r="1730"/>
+    <row r="1731"/>
+    <row r="1732"/>
+    <row r="1733"/>
+    <row r="1734"/>
+    <row r="1735"/>
+    <row r="1736"/>
+    <row r="1737"/>
+    <row r="1738"/>
+    <row r="1739"/>
+    <row r="1740"/>
+    <row r="1741"/>
+    <row r="1742"/>
+    <row r="1743"/>
+    <row r="1744"/>
+    <row r="1745"/>
+    <row r="1746"/>
+    <row r="1747"/>
+    <row r="1748"/>
+    <row r="1749"/>
+    <row r="1750"/>
+    <row r="1751"/>
+    <row r="1752"/>
+    <row r="1753"/>
+    <row r="1754"/>
+    <row r="1755"/>
+    <row r="1756"/>
+    <row r="1757"/>
+    <row r="1758"/>
+    <row r="1759"/>
+    <row r="1760"/>
+    <row r="1761"/>
+    <row r="1762"/>
+    <row r="1763"/>
+    <row r="1764"/>
+    <row r="1765"/>
+    <row r="1766"/>
+    <row r="1767"/>
+    <row r="1768"/>
+    <row r="1769"/>
+    <row r="1770"/>
+    <row r="1771"/>
+    <row r="1772"/>
+    <row r="1773"/>
+    <row r="1774"/>
+    <row r="1775"/>
+    <row r="1776"/>
+    <row r="1777"/>
+    <row r="1778"/>
+    <row r="1779"/>
+    <row r="1780"/>
+    <row r="1781"/>
+    <row r="1782"/>
+    <row r="1783"/>
+    <row r="1784"/>
+    <row r="1785"/>
+    <row r="1786"/>
+    <row r="1787"/>
+    <row r="1788"/>
+    <row r="1789"/>
+    <row r="1790"/>
+    <row r="1791"/>
+    <row r="1792"/>
+    <row r="1793"/>
+    <row r="1794"/>
+    <row r="1795"/>
+    <row r="1796"/>
+    <row r="1797"/>
+    <row r="1798"/>
+    <row r="1799"/>
+    <row r="1800"/>
+    <row r="1801"/>
+    <row r="1802"/>
+    <row r="1803"/>
+    <row r="1804"/>
+    <row r="1805"/>
+    <row r="1806"/>
+    <row r="1807"/>
+    <row r="1808"/>
+    <row r="1809"/>
+    <row r="1810"/>
+    <row r="1811"/>
+    <row r="1812"/>
+    <row r="1813"/>
+    <row r="1814"/>
+    <row r="1815"/>
+    <row r="1816"/>
+    <row r="1817"/>
+    <row r="1818"/>
+    <row r="1819"/>
+    <row r="1820"/>
+    <row r="1821"/>
+    <row r="1822"/>
+    <row r="1823"/>
+    <row r="1824"/>
+    <row r="1825"/>
+    <row r="1826"/>
+    <row r="1827"/>
+    <row r="1828"/>
+    <row r="1829"/>
+    <row r="1830"/>
+    <row r="1831"/>
+    <row r="1832"/>
+    <row r="1833"/>
+    <row r="1834"/>
+    <row r="1835"/>
+    <row r="1836"/>
+    <row r="1837"/>
+    <row r="1838"/>
+    <row r="1839"/>
+    <row r="1840"/>
+    <row r="1841"/>
+    <row r="1842"/>
+    <row r="1843"/>
+    <row r="1844"/>
+    <row r="1845"/>
+    <row r="1846"/>
+    <row r="1847"/>
+    <row r="1848"/>
+    <row r="1849"/>
+    <row r="1850"/>
+    <row r="1851"/>
+    <row r="1852"/>
+    <row r="1853"/>
+    <row r="1854"/>
+    <row r="1855"/>
+    <row r="1856"/>
+    <row r="1857"/>
+    <row r="1858"/>
+    <row r="1859"/>
+    <row r="1860"/>
+    <row r="1861"/>
+    <row r="1862"/>
     <row r="1863" ht="15" customHeight="1"/>
     <row r="1864" ht="15" customHeight="1"/>
     <row r="1865" ht="15" customHeight="1"/>
@@ -72797,9 +73097,6 @@
       <c r="H2491" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2491" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2492">
       <c r="A2492" t="inlineStr">
@@ -72836,9 +73133,6 @@
       <c r="H2492" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2492" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2493">
       <c r="A2493" t="inlineStr">
@@ -72875,9 +73169,6 @@
       <c r="H2493" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2493" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2494">
       <c r="A2494" t="inlineStr">
@@ -72914,9 +73205,6 @@
       <c r="H2494" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2494" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2495">
       <c r="A2495" t="inlineStr">
@@ -72953,9 +73241,6 @@
       <c r="H2495" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2495" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2496">
       <c r="A2496" t="inlineStr">
@@ -72992,9 +73277,6 @@
       <c r="H2496" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2496" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2497">
       <c r="A2497" t="inlineStr">
@@ -73031,9 +73313,6 @@
       <c r="H2497" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2497" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2498">
       <c r="A2498" t="inlineStr">
@@ -73148,9 +73427,6 @@
       <c r="H2500" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2500" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2501">
       <c r="A2501" t="inlineStr">
@@ -73226,9 +73502,6 @@
       <c r="H2502" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2502" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2503">
       <c r="A2503" t="inlineStr">
@@ -73265,9 +73538,6 @@
       <c r="H2503" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2503" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2504">
       <c r="A2504" t="inlineStr">
@@ -73304,9 +73574,6 @@
       <c r="H2504" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2504" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2505">
       <c r="A2505" t="inlineStr">
@@ -73343,9 +73610,6 @@
       <c r="H2505" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2505" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2506">
       <c r="A2506" t="inlineStr">
@@ -73382,9 +73646,6 @@
       <c r="H2506" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2506" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2507">
       <c r="A2507" t="inlineStr">
@@ -73421,9 +73682,6 @@
       <c r="H2507" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2507" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2508">
       <c r="A2508" t="inlineStr">
@@ -73460,9 +73718,6 @@
       <c r="H2508" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2508" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2509">
       <c r="A2509" t="inlineStr">
@@ -73499,9 +73754,6 @@
       <c r="H2509" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2509" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2510">
       <c r="A2510" t="inlineStr">
@@ -73538,9 +73790,6 @@
       <c r="H2510" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2510" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2511">
       <c r="A2511" t="inlineStr">
@@ -73616,9 +73865,6 @@
       <c r="H2512" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2512" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2513">
       <c r="A2513" t="inlineStr">
@@ -73655,9 +73901,6 @@
       <c r="H2513" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2513" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2514">
       <c r="A2514" t="inlineStr">
@@ -73733,9 +73976,6 @@
       <c r="H2515" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2515" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2516">
       <c r="A2516" t="inlineStr">
@@ -73772,9 +74012,6 @@
       <c r="H2516" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2516" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2517">
       <c r="A2517" t="inlineStr">
@@ -73811,9 +74048,6 @@
       <c r="H2517" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2517" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2518">
       <c r="A2518" t="inlineStr">
@@ -73850,9 +74084,6 @@
       <c r="H2518" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2518" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2519">
       <c r="A2519" t="inlineStr">
@@ -73889,9 +74120,6 @@
       <c r="H2519" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2519" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2520">
       <c r="A2520" t="inlineStr">
@@ -73967,9 +74195,6 @@
       <c r="H2521" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2521" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2522">
       <c r="A2522" t="inlineStr">
@@ -74006,9 +74231,6 @@
       <c r="H2522" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2522" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2523">
       <c r="A2523" t="inlineStr">
@@ -74081,9 +74303,6 @@
       <c r="H2524" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2524" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2525">
       <c r="A2525" t="inlineStr">
@@ -74156,9 +74375,6 @@
       <c r="H2526" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2526" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2527">
       <c r="A2527" t="inlineStr">
@@ -74312,9 +74528,6 @@
       <c r="H2530" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2530" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2531">
       <c r="A2531" t="inlineStr">
@@ -74351,9 +74564,6 @@
       <c r="H2531" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2531" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2532">
       <c r="A2532" t="inlineStr">
@@ -74390,9 +74600,6 @@
       <c r="H2532" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2532" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2533">
       <c r="A2533" t="inlineStr">
@@ -74507,9 +74714,6 @@
       <c r="H2535" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2535" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2536">
       <c r="A2536" t="inlineStr">
@@ -74585,9 +74789,6 @@
       <c r="H2537" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2537" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2538">
       <c r="A2538" t="inlineStr">
@@ -74624,9 +74825,6 @@
       <c r="H2538" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2538" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2539">
       <c r="A2539" t="inlineStr">
@@ -74634,9 +74832,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2539" t="n">
-        <v/>
-      </c>
       <c r="C2539" t="inlineStr">
         <is>
           <t>https://www.hoogvliet.com/product/vis-marine-wilde-zalm</t>
@@ -74702,9 +74897,6 @@
       <c r="H2540" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2540" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2541">
       <c r="A2541" t="inlineStr">
@@ -74712,9 +74904,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2541" t="n">
-        <v/>
-      </c>
       <c r="C2541" t="inlineStr">
         <is>
           <t>https://www.hoogvliet.com/product/vis-marine-kabeljauwfilets</t>
@@ -74741,9 +74930,6 @@
       <c r="H2541" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2541" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2542">
       <c r="A2542" t="inlineStr">
@@ -74780,9 +74966,6 @@
       <c r="H2542" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2542" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2543">
       <c r="A2543" t="inlineStr">
@@ -74819,9 +75002,6 @@
       <c r="H2543" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2543" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2544">
       <c r="A2544" t="inlineStr">
@@ -74858,9 +75038,6 @@
       <c r="H2544" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2544" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2545">
       <c r="A2545" t="inlineStr">
@@ -74897,9 +75074,6 @@
       <c r="H2545" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2545" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2546">
       <c r="A2546" t="inlineStr">
@@ -74936,9 +75110,6 @@
       <c r="H2546" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2546" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2547">
       <c r="A2547" t="inlineStr">
@@ -74946,9 +75117,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2547" t="n">
-        <v/>
-      </c>
       <c r="C2547" t="inlineStr">
         <is>
           <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/vis%20marine%20koolvisfilet%204%20stuks/49562</t>
@@ -74975,9 +75143,6 @@
       <c r="H2547" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2547" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2548">
       <c r="A2548" t="inlineStr">
@@ -74985,9 +75150,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2548" t="n">
-        <v/>
-      </c>
       <c r="C2548" t="inlineStr">
         <is>
           <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/vis%20marine%20kabeljauwfilet%204%20stuks/49672</t>
@@ -75014,9 +75176,6 @@
       <c r="H2548" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2548" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2549">
       <c r="A2549" t="inlineStr">
@@ -75024,9 +75183,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2549" t="n">
-        <v/>
-      </c>
       <c r="C2549" t="inlineStr">
         <is>
           <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/vis%20marine%20pangasiusfilet/82503</t>
@@ -75063,9 +75219,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2550" t="n">
-        <v/>
-      </c>
       <c r="C2550" t="inlineStr">
         <is>
           <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/vis%20marine%20wilde%20zalm/96927</t>
@@ -75102,9 +75255,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2551" t="n">
-        <v/>
-      </c>
       <c r="C2551" t="inlineStr">
         <is>
           <t>https://www.plus.nl/product/vis-marine-koolvisfilets-doos-400-g-834796</t>
@@ -75131,9 +75281,6 @@
       <c r="H2551" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2551" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2552">
       <c r="A2552" t="inlineStr">
@@ -75170,9 +75317,6 @@
       <c r="H2552" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2552" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2553">
       <c r="A2553" t="inlineStr">
@@ -75180,9 +75324,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2553" t="n">
-        <v/>
-      </c>
       <c r="C2553" t="inlineStr">
         <is>
           <t>https://www.spar.nl/vis-marine-kabeljauwfilets-4-stuks-9228133/</t>
@@ -75209,9 +75350,6 @@
       <c r="H2553" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2553" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2554">
       <c r="A2554" t="inlineStr">
@@ -75219,9 +75357,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2554" t="n">
-        <v/>
-      </c>
       <c r="C2554" t="inlineStr">
         <is>
           <t>https://www.spar.nl/vis-marine-pangasius-filets-9188805/</t>
@@ -75258,9 +75393,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2555" t="n">
-        <v/>
-      </c>
       <c r="C2555" t="inlineStr">
         <is>
           <t>https://www.spar.nl/vis-marine-wilde-zalmfilet-9194254/</t>
@@ -75297,9 +75429,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2556" t="n">
-        <v/>
-      </c>
       <c r="C2556" t="inlineStr">
         <is>
           <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307411</t>
@@ -75326,9 +75455,6 @@
       <c r="H2556" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2556" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2557">
       <c r="A2557" t="inlineStr">
@@ -75336,9 +75462,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2557" t="n">
-        <v/>
-      </c>
       <c r="C2557" t="inlineStr">
         <is>
           <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307028</t>
@@ -75375,9 +75498,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2558" t="n">
-        <v/>
-      </c>
       <c r="C2558" t="inlineStr">
         <is>
           <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307026</t>
@@ -75414,9 +75534,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2559" t="n">
-        <v/>
-      </c>
       <c r="C2559" t="inlineStr">
         <is>
           <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307023</t>
@@ -75453,9 +75570,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2560" t="n">
-        <v/>
-      </c>
       <c r="C2560" t="inlineStr">
         <is>
           <t>https://www.hoogvliet.com/product/vis-marine-koolvisfilets</t>
@@ -75482,9 +75596,6 @@
       <c r="H2560" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2560" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2561">
       <c r="A2561" t="inlineStr">
@@ -75492,9 +75603,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2561" t="n">
-        <v/>
-      </c>
       <c r="C2561" t="inlineStr">
         <is>
           <t>https://www.plus.nl/product/plus-tilapiafilets-zak-540-g-793166?utm_source=awin&amp;utm_medium=affiliate&amp;utm_campaign=531573_ShopForward+CSS&amp;utm_content=0&amp;sv1=affiliate&amp;sv_campaign_id=531573&amp;awc=12479_1776164499_4fdb47ad85457250f177963ef4cdf5d9</t>
@@ -75506,7 +75614,7 @@
         </is>
       </c>
       <c r="E2561" t="n">
-        <v>496.45</v>
+        <v>6.45</v>
       </c>
       <c r="F2561" t="inlineStr">
         <is>
@@ -75521,9 +75629,6 @@
       <c r="H2561" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2561" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2562">
       <c r="A2562" t="inlineStr">
@@ -75560,9 +75665,6 @@
       <c r="H2562" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2562" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2563">
       <c r="A2563" t="inlineStr">
@@ -75570,9 +75672,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2563" t="n">
-        <v/>
-      </c>
       <c r="C2563" t="inlineStr">
         <is>
           <t>https://www.plus.nl/product/vis-marine-kabeljauwfilets-msc-doos-540-g-723219</t>
@@ -75638,9 +75737,6 @@
       <c r="H2564" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2564" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2565">
       <c r="A2565" t="inlineStr">
@@ -75648,9 +75744,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2565" t="n">
-        <v/>
-      </c>
       <c r="C2565" t="inlineStr">
         <is>
           <t>https://www.aldi.nl/product/wilde-zalmfilets-1204877.html</t>
@@ -75716,9 +75809,6 @@
       <c r="H2566" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2566" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2567">
       <c r="A2567" t="inlineStr">
@@ -75726,9 +75816,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2567" t="n">
-        <v/>
-      </c>
       <c r="C2567" t="inlineStr">
         <is>
           <t>https://www.jumbo.com/producten/jumbo-zalmfilet-met-huid-2-x-125-g-723226DS</t>
@@ -75755,9 +75842,6 @@
       <c r="H2567" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2567" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2568">
       <c r="A2568" t="inlineStr">
@@ -75765,9 +75849,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2568" t="n">
-        <v/>
-      </c>
       <c r="C2568" t="inlineStr">
         <is>
           <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis%20marine%20koolvisfilet%204%20stuks/49562</t>
@@ -75794,9 +75875,6 @@
       <c r="H2568" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2568" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2569">
       <c r="A2569" t="inlineStr">
@@ -75804,9 +75882,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2569" t="n">
-        <v/>
-      </c>
       <c r="C2569" t="inlineStr">
         <is>
           <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis%20marine%20kabeljauwfilets/111544</t>
@@ -75840,9 +75915,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2570" t="n">
-        <v/>
-      </c>
       <c r="C2570" t="inlineStr">
         <is>
           <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis%20marine%20pangasiusfilet/82503</t>
@@ -75879,9 +75951,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2571" t="n">
-        <v/>
-      </c>
       <c r="C2571" t="inlineStr">
         <is>
           <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis%20marine%20wilde%20zalm/96927</t>
@@ -75918,9 +75987,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2572" t="n">
-        <v/>
-      </c>
       <c r="C2572" t="inlineStr">
         <is>
           <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis-marine-tilapia-filets-5-6-st/83124</t>
@@ -75947,9 +76013,6 @@
       <c r="H2572" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2572" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2573">
       <c r="A2573" t="inlineStr">
@@ -75957,9 +76020,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2573" t="n">
-        <v/>
-      </c>
       <c r="C2573" t="inlineStr">
         <is>
           <t>https://www.jumbo.com/producten/jumbo-koolvis-filet-400-g-713748DS</t>
@@ -75986,9 +76046,6 @@
       <c r="H2573" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2573" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2574">
       <c r="A2574" t="inlineStr">
@@ -75996,9 +76053,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2574" t="n">
-        <v/>
-      </c>
       <c r="C2574" t="inlineStr">
         <is>
           <t>https://www.jumbo.com/producten/seacon-alaska-koolvisfilet-675g-706749ZK</t>
@@ -76035,9 +76089,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2575" t="n">
-        <v/>
-      </c>
       <c r="C2575" t="inlineStr">
         <is>
           <t>https://www.jumbo.com/producten/jumbo-kabeljauwfilet-675-g-471158ZK</t>
@@ -76074,9 +76125,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2576" t="n">
-        <v/>
-      </c>
       <c r="C2576" t="inlineStr">
         <is>
           <t>https://www.jumbo.com/producten/jumbo-pangasiusfilet-vriesvers-675-g-494433ZK</t>
@@ -76113,9 +76161,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2577" t="n">
-        <v/>
-      </c>
       <c r="C2577" t="inlineStr">
         <is>
           <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/vismarine-pangasiusfilet-540gr/110960</t>
@@ -76152,9 +76197,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2578" t="n">
-        <v/>
-      </c>
       <c r="C2578" t="inlineStr">
         <is>
           <t>https://www.jumbo.com/producten/jumbo-pangasiusfilet-270-g-173837ZK</t>
@@ -76181,9 +76223,6 @@
       <c r="H2578" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2578" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2579">
       <c r="A2579" t="inlineStr">
@@ -76191,9 +76230,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2579" t="n">
-        <v/>
-      </c>
       <c r="C2579" t="inlineStr">
         <is>
           <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/vismarine-koolvisfilet-4stmsc/811408</t>
@@ -76220,9 +76256,6 @@
       <c r="H2579" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2579" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2580">
       <c r="A2580" t="inlineStr">
@@ -76230,9 +76263,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2580" t="n">
-        <v/>
-      </c>
       <c r="C2580" t="inlineStr">
         <is>
           <t>https://www.jumbo.com/producten/jumbo-wilde-zalmfilet-2-x-125-g-76159PAK</t>
@@ -76259,9 +76289,6 @@
       <c r="H2580" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2580" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2581">
       <c r="A2581" t="inlineStr">
@@ -76269,9 +76296,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2581" t="n">
-        <v/>
-      </c>
       <c r="C2581" t="inlineStr">
         <is>
           <t>https://www.ah.nl/producten/product/wi39826/ah-koolvisfilet</t>
@@ -76298,9 +76322,6 @@
       <c r="H2581" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2581" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2582">
       <c r="A2582" t="inlineStr">
@@ -76308,9 +76329,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2582" t="n">
-        <v/>
-      </c>
       <c r="C2582" t="inlineStr">
         <is>
           <t>https://www.ah.nl/producten/product/wi121478/ah-kabeljauwfilet</t>
@@ -76347,9 +76365,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2583" t="n">
-        <v/>
-      </c>
       <c r="C2583" t="inlineStr">
         <is>
           <t>https://www.ah.nl/producten/product/wi792/ah-kabeljauw</t>
@@ -76376,9 +76391,6 @@
       <c r="H2583" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2583" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2584">
       <c r="A2584" t="inlineStr">
@@ -76386,9 +76398,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2584" t="n">
-        <v/>
-      </c>
       <c r="C2584" t="inlineStr">
         <is>
           <t>https://www.ah.nl/producten/product/wi140671/ah-pangasiusfilet</t>
@@ -76425,9 +76434,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2585" t="n">
-        <v/>
-      </c>
       <c r="C2585" t="inlineStr">
         <is>
           <t>https://www.ah.nl/producten/product/wi141565/ah-wilde-zalmfilets</t>
@@ -76464,9 +76470,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2586" t="n">
-        <v/>
-      </c>
       <c r="C2586" t="inlineStr">
         <is>
           <t>https://www.ah.nl/producten/product/wi178129/ah-wilde-zalmfilet</t>
@@ -76493,9 +76496,6 @@
       <c r="H2586" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2586" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2587">
       <c r="A2587" t="inlineStr">
@@ -76503,9 +76503,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2587" t="n">
-        <v/>
-      </c>
       <c r="C2587" t="inlineStr">
         <is>
           <t>https://www.ah.nl/producten/product/wi396815/ah-tilapiafilet-graatvrij</t>
@@ -76532,9 +76529,6 @@
       <c r="H2587" s="13" t="n">
         <v>46160</v>
       </c>
-      <c r="I2587" t="n">
-        <v/>
-      </c>
     </row>
     <row r="2588">
       <c r="A2588" t="inlineStr">
@@ -76542,9 +76536,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2588" t="n">
-        <v/>
-      </c>
       <c r="C2588" t="inlineStr">
         <is>
           <t>https://www.aldi.nl/product/pangasiusfilet-1221684.html</t>
@@ -76581,9 +76572,6 @@
           <t>Concurrent</t>
         </is>
       </c>
-      <c r="B2589" t="n">
-        <v/>
-      </c>
       <c r="C2589" t="inlineStr">
         <is>
           <t>https://www.jumbo.com/producten/jumbo-wilde-zalm-filet-675-g-487780ZK</t>
@@ -76648,9 +76636,6 @@
       </c>
       <c r="H2590" s="13" t="n">
         <v>46160</v>
-      </c>
-      <c r="I2590" t="n">
-        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
URL Plus Tilapia opgeschoond (tracking parameters verwijderd)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -63239,7 +63239,7 @@
       </c>
       <c r="C1305" t="inlineStr">
         <is>
-          <t>https://www.plus.nl/product/plus-tilapiafilets-zak-540-g-793166?utm_source=awin&amp;utm_medium=affiliate&amp;utm_campaign=531573_ShopForward+CSS&amp;utm_content=0&amp;sv1=affiliate&amp;sv_campaign_id=531573&amp;awc=12479_1776164499_4fdb47ad85457250f177963ef4cdf5d9</t>
+          <t>https://www.plus.nl/product/plus-tilapiafilets-zak-540-g-793166</t>
         </is>
       </c>
       <c r="D1305" t="inlineStr">
@@ -66755,7 +66755,7 @@
       </c>
       <c r="C1403" t="inlineStr">
         <is>
-          <t>https://www.plus.nl/product/plus-tilapiafilets-zak-540-g-793166?utm_source=awin&amp;utm_medium=affiliate&amp;utm_campaign=531573_ShopForward+CSS&amp;utm_content=0&amp;sv1=affiliate&amp;sv_campaign_id=531573&amp;awc=12479_1776164499_4fdb47ad85457250f177963ef4cdf5d9</t>
+          <t>https://www.plus.nl/product/plus-tilapiafilets-zak-540-g-793166</t>
         </is>
       </c>
       <c r="D1403" t="inlineStr">
@@ -68222,7 +68222,7 @@
       </c>
       <c r="C1445" t="inlineStr">
         <is>
-          <t>https://www.plus.nl/product/plus-tilapiafilets-zak-540-g-793166?utm_source=awin&amp;utm_medium=affiliate&amp;utm_campaign=531573_ShopForward+CSS&amp;utm_content=0&amp;sv1=affiliate&amp;sv_campaign_id=531573&amp;awc=12479_1776164499_4fdb47ad85457250f177963ef4cdf5d9</t>
+          <t>https://www.plus.nl/product/plus-tilapiafilets-zak-540-g-793166</t>
         </is>
       </c>
       <c r="D1445" t="inlineStr">
@@ -75605,7 +75605,7 @@
       </c>
       <c r="C2561" t="inlineStr">
         <is>
-          <t>https://www.plus.nl/product/plus-tilapiafilets-zak-540-g-793166?utm_source=awin&amp;utm_medium=affiliate&amp;utm_campaign=531573_ShopForward+CSS&amp;utm_content=0&amp;sv1=affiliate&amp;sv_campaign_id=531573&amp;awc=12479_1776164499_4fdb47ad85457250f177963ef4cdf5d9</t>
+          <t>https://www.plus.nl/product/plus-tilapiafilets-zak-540-g-793166</t>
         </is>
       </c>
       <c r="D2561" t="inlineStr">

</xml_diff>

<commit_message>
Nieuw product toegevoegd via app - 2026-05-21
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -17238,7 +17238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2590"/>
+  <dimension ref="A1:I2591"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="20.140625" customWidth="1" min="1" max="1"/>
@@ -71847,306 +71847,6 @@
     <row r="1562" ht="15" customHeight="1">
       <c r="H1562" s="1" t="n"/>
     </row>
-    <row r="1563"/>
-    <row r="1564"/>
-    <row r="1565"/>
-    <row r="1566"/>
-    <row r="1567"/>
-    <row r="1568"/>
-    <row r="1569"/>
-    <row r="1570"/>
-    <row r="1571"/>
-    <row r="1572"/>
-    <row r="1573"/>
-    <row r="1574"/>
-    <row r="1575"/>
-    <row r="1576"/>
-    <row r="1577"/>
-    <row r="1578"/>
-    <row r="1579"/>
-    <row r="1580"/>
-    <row r="1581"/>
-    <row r="1582"/>
-    <row r="1583"/>
-    <row r="1584"/>
-    <row r="1585"/>
-    <row r="1586"/>
-    <row r="1587"/>
-    <row r="1588"/>
-    <row r="1589"/>
-    <row r="1590"/>
-    <row r="1591"/>
-    <row r="1592"/>
-    <row r="1593"/>
-    <row r="1594"/>
-    <row r="1595"/>
-    <row r="1596"/>
-    <row r="1597"/>
-    <row r="1598"/>
-    <row r="1599"/>
-    <row r="1600"/>
-    <row r="1601"/>
-    <row r="1602"/>
-    <row r="1603"/>
-    <row r="1604"/>
-    <row r="1605"/>
-    <row r="1606"/>
-    <row r="1607"/>
-    <row r="1608"/>
-    <row r="1609"/>
-    <row r="1610"/>
-    <row r="1611"/>
-    <row r="1612"/>
-    <row r="1613"/>
-    <row r="1614"/>
-    <row r="1615"/>
-    <row r="1616"/>
-    <row r="1617"/>
-    <row r="1618"/>
-    <row r="1619"/>
-    <row r="1620"/>
-    <row r="1621"/>
-    <row r="1622"/>
-    <row r="1623"/>
-    <row r="1624"/>
-    <row r="1625"/>
-    <row r="1626"/>
-    <row r="1627"/>
-    <row r="1628"/>
-    <row r="1629"/>
-    <row r="1630"/>
-    <row r="1631"/>
-    <row r="1632"/>
-    <row r="1633"/>
-    <row r="1634"/>
-    <row r="1635"/>
-    <row r="1636"/>
-    <row r="1637"/>
-    <row r="1638"/>
-    <row r="1639"/>
-    <row r="1640"/>
-    <row r="1641"/>
-    <row r="1642"/>
-    <row r="1643"/>
-    <row r="1644"/>
-    <row r="1645"/>
-    <row r="1646"/>
-    <row r="1647"/>
-    <row r="1648"/>
-    <row r="1649"/>
-    <row r="1650"/>
-    <row r="1651"/>
-    <row r="1652"/>
-    <row r="1653"/>
-    <row r="1654"/>
-    <row r="1655"/>
-    <row r="1656"/>
-    <row r="1657"/>
-    <row r="1658"/>
-    <row r="1659"/>
-    <row r="1660"/>
-    <row r="1661"/>
-    <row r="1662"/>
-    <row r="1663"/>
-    <row r="1664"/>
-    <row r="1665"/>
-    <row r="1666"/>
-    <row r="1667"/>
-    <row r="1668"/>
-    <row r="1669"/>
-    <row r="1670"/>
-    <row r="1671"/>
-    <row r="1672"/>
-    <row r="1673"/>
-    <row r="1674"/>
-    <row r="1675"/>
-    <row r="1676"/>
-    <row r="1677"/>
-    <row r="1678"/>
-    <row r="1679"/>
-    <row r="1680"/>
-    <row r="1681"/>
-    <row r="1682"/>
-    <row r="1683"/>
-    <row r="1684"/>
-    <row r="1685"/>
-    <row r="1686"/>
-    <row r="1687"/>
-    <row r="1688"/>
-    <row r="1689"/>
-    <row r="1690"/>
-    <row r="1691"/>
-    <row r="1692"/>
-    <row r="1693"/>
-    <row r="1694"/>
-    <row r="1695"/>
-    <row r="1696"/>
-    <row r="1697"/>
-    <row r="1698"/>
-    <row r="1699"/>
-    <row r="1700"/>
-    <row r="1701"/>
-    <row r="1702"/>
-    <row r="1703"/>
-    <row r="1704"/>
-    <row r="1705"/>
-    <row r="1706"/>
-    <row r="1707"/>
-    <row r="1708"/>
-    <row r="1709"/>
-    <row r="1710"/>
-    <row r="1711"/>
-    <row r="1712"/>
-    <row r="1713"/>
-    <row r="1714"/>
-    <row r="1715"/>
-    <row r="1716"/>
-    <row r="1717"/>
-    <row r="1718"/>
-    <row r="1719"/>
-    <row r="1720"/>
-    <row r="1721"/>
-    <row r="1722"/>
-    <row r="1723"/>
-    <row r="1724"/>
-    <row r="1725"/>
-    <row r="1726"/>
-    <row r="1727"/>
-    <row r="1728"/>
-    <row r="1729"/>
-    <row r="1730"/>
-    <row r="1731"/>
-    <row r="1732"/>
-    <row r="1733"/>
-    <row r="1734"/>
-    <row r="1735"/>
-    <row r="1736"/>
-    <row r="1737"/>
-    <row r="1738"/>
-    <row r="1739"/>
-    <row r="1740"/>
-    <row r="1741"/>
-    <row r="1742"/>
-    <row r="1743"/>
-    <row r="1744"/>
-    <row r="1745"/>
-    <row r="1746"/>
-    <row r="1747"/>
-    <row r="1748"/>
-    <row r="1749"/>
-    <row r="1750"/>
-    <row r="1751"/>
-    <row r="1752"/>
-    <row r="1753"/>
-    <row r="1754"/>
-    <row r="1755"/>
-    <row r="1756"/>
-    <row r="1757"/>
-    <row r="1758"/>
-    <row r="1759"/>
-    <row r="1760"/>
-    <row r="1761"/>
-    <row r="1762"/>
-    <row r="1763"/>
-    <row r="1764"/>
-    <row r="1765"/>
-    <row r="1766"/>
-    <row r="1767"/>
-    <row r="1768"/>
-    <row r="1769"/>
-    <row r="1770"/>
-    <row r="1771"/>
-    <row r="1772"/>
-    <row r="1773"/>
-    <row r="1774"/>
-    <row r="1775"/>
-    <row r="1776"/>
-    <row r="1777"/>
-    <row r="1778"/>
-    <row r="1779"/>
-    <row r="1780"/>
-    <row r="1781"/>
-    <row r="1782"/>
-    <row r="1783"/>
-    <row r="1784"/>
-    <row r="1785"/>
-    <row r="1786"/>
-    <row r="1787"/>
-    <row r="1788"/>
-    <row r="1789"/>
-    <row r="1790"/>
-    <row r="1791"/>
-    <row r="1792"/>
-    <row r="1793"/>
-    <row r="1794"/>
-    <row r="1795"/>
-    <row r="1796"/>
-    <row r="1797"/>
-    <row r="1798"/>
-    <row r="1799"/>
-    <row r="1800"/>
-    <row r="1801"/>
-    <row r="1802"/>
-    <row r="1803"/>
-    <row r="1804"/>
-    <row r="1805"/>
-    <row r="1806"/>
-    <row r="1807"/>
-    <row r="1808"/>
-    <row r="1809"/>
-    <row r="1810"/>
-    <row r="1811"/>
-    <row r="1812"/>
-    <row r="1813"/>
-    <row r="1814"/>
-    <row r="1815"/>
-    <row r="1816"/>
-    <row r="1817"/>
-    <row r="1818"/>
-    <row r="1819"/>
-    <row r="1820"/>
-    <row r="1821"/>
-    <row r="1822"/>
-    <row r="1823"/>
-    <row r="1824"/>
-    <row r="1825"/>
-    <row r="1826"/>
-    <row r="1827"/>
-    <row r="1828"/>
-    <row r="1829"/>
-    <row r="1830"/>
-    <row r="1831"/>
-    <row r="1832"/>
-    <row r="1833"/>
-    <row r="1834"/>
-    <row r="1835"/>
-    <row r="1836"/>
-    <row r="1837"/>
-    <row r="1838"/>
-    <row r="1839"/>
-    <row r="1840"/>
-    <row r="1841"/>
-    <row r="1842"/>
-    <row r="1843"/>
-    <row r="1844"/>
-    <row r="1845"/>
-    <row r="1846"/>
-    <row r="1847"/>
-    <row r="1848"/>
-    <row r="1849"/>
-    <row r="1850"/>
-    <row r="1851"/>
-    <row r="1852"/>
-    <row r="1853"/>
-    <row r="1854"/>
-    <row r="1855"/>
-    <row r="1856"/>
-    <row r="1857"/>
-    <row r="1858"/>
-    <row r="1859"/>
-    <row r="1860"/>
-    <row r="1861"/>
-    <row r="1862"/>
     <row r="1863" ht="15" customHeight="1"/>
     <row r="1864" ht="15" customHeight="1"/>
     <row r="1865" ht="15" customHeight="1"/>
@@ -76638,6 +76338,42 @@
         <v>46160</v>
       </c>
     </row>
+    <row r="2591">
+      <c r="A2591" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2591" t="n">
+        <v>17025</v>
+      </c>
+      <c r="C2591" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi599401/ah-ijs-spinners</t>
+        </is>
+      </c>
+      <c r="D2591" t="inlineStr">
+        <is>
+          <t>AH SPINNER AARDBEI SINAASAPPEL VANILLE</t>
+        </is>
+      </c>
+      <c r="E2591" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="F2591" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2591" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2591" s="13" t="n">
+        <v>46163</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId1"/>

</xml_diff>

<commit_message>
Data update di 26-05-2026
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -17238,7 +17238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2595"/>
+  <dimension ref="A1:I2698"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="20.140625" customWidth="1" min="1" max="1"/>
@@ -76518,6 +76518,4008 @@
         <v>46163</v>
       </c>
     </row>
+    <row r="2596">
+      <c r="A2596" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2596" t="n">
+        <v/>
+      </c>
+      <c r="C2596" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-wilde-zalm-filet-675-g-487780ZK</t>
+        </is>
+      </c>
+      <c r="D2596" t="inlineStr">
+        <is>
+          <t>Jumbo Wilde Zalm Filet 675g</t>
+        </is>
+      </c>
+      <c r="E2596" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="F2596" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2596" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2596" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2596" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2597">
+      <c r="A2597" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2597" t="n">
+        <v>27300</v>
+      </c>
+      <c r="C2597" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-brood-bladerdeeg/knoflookbaguette-175gr/301172</t>
+        </is>
+      </c>
+      <c r="D2597" t="inlineStr">
+        <is>
+          <t>KNOFLOOKBAGUETTE</t>
+        </is>
+      </c>
+      <c r="E2597" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="F2597" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2597" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2597" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2597" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2598">
+      <c r="A2598" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2598" t="n">
+        <v>27704</v>
+      </c>
+      <c r="C2598" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/528-ijsballen-zak-1-kg-769217</t>
+        </is>
+      </c>
+      <c r="D2598" t="inlineStr">
+        <is>
+          <t>528 ICE BALLS 1KG</t>
+        </is>
+      </c>
+      <c r="E2598" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="F2598" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2598" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2598" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2598" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2599">
+      <c r="A2599" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2599" t="n">
+        <v/>
+      </c>
+      <c r="C2599" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/plus-tilapiafilets-zak-540-g-793166</t>
+        </is>
+      </c>
+      <c r="D2599" t="inlineStr">
+        <is>
+          <t>Plus Tilapiafilets 540g</t>
+        </is>
+      </c>
+      <c r="E2599" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="F2599" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2599" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2599" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2599" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2600">
+      <c r="A2600" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2600" t="n">
+        <v/>
+      </c>
+      <c r="C2600" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/vis-marine-koolvisfilets</t>
+        </is>
+      </c>
+      <c r="D2600" t="inlineStr">
+        <is>
+          <t>Vis Marine Koolvis 400g</t>
+        </is>
+      </c>
+      <c r="E2600" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F2600" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2600" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2600" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2600" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2601">
+      <c r="A2601" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2601" t="n">
+        <v/>
+      </c>
+      <c r="C2601" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307023</t>
+        </is>
+      </c>
+      <c r="D2601" t="inlineStr">
+        <is>
+          <t>Vis Marine Wilde zalm 540g</t>
+        </is>
+      </c>
+      <c r="E2601" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F2601" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2601" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2601" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2601" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2602">
+      <c r="A2602" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2602" t="n">
+        <v/>
+      </c>
+      <c r="C2602" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307026</t>
+        </is>
+      </c>
+      <c r="D2602" t="inlineStr">
+        <is>
+          <t>Vis Marine Pangasiusfilet 540g</t>
+        </is>
+      </c>
+      <c r="E2602" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="F2602" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2602" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2602" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2602" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2603">
+      <c r="A2603" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2603" t="n">
+        <v/>
+      </c>
+      <c r="C2603" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307028</t>
+        </is>
+      </c>
+      <c r="D2603" t="inlineStr">
+        <is>
+          <t>Vis Marine Kabeljauw 540g</t>
+        </is>
+      </c>
+      <c r="E2603" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="F2603" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2603" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2603" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2603" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2604">
+      <c r="A2604" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2604" t="n">
+        <v/>
+      </c>
+      <c r="C2604" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307411</t>
+        </is>
+      </c>
+      <c r="D2604" t="inlineStr">
+        <is>
+          <t>Vis Marine Koolvis 400g</t>
+        </is>
+      </c>
+      <c r="E2604" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="F2604" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2604" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2604" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2604" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2605">
+      <c r="A2605" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2605" t="n">
+        <v/>
+      </c>
+      <c r="C2605" t="inlineStr">
+        <is>
+          <t>https://www.spar.nl/vis-marine-wilde-zalmfilet-9194254/</t>
+        </is>
+      </c>
+      <c r="D2605" t="inlineStr">
+        <is>
+          <t>Vis Marine Wilde zalm 540g</t>
+        </is>
+      </c>
+      <c r="E2605" t="n">
+        <v>6.59</v>
+      </c>
+      <c r="F2605" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="G2605" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2605" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2605" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2606">
+      <c r="A2606" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2606" t="n">
+        <v/>
+      </c>
+      <c r="C2606" t="inlineStr">
+        <is>
+          <t>https://www.spar.nl/vis-marine-pangasius-filets-9188805/</t>
+        </is>
+      </c>
+      <c r="D2606" t="inlineStr">
+        <is>
+          <t>Vis Marine Pangasiusfilet 540g</t>
+        </is>
+      </c>
+      <c r="E2606" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F2606" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="G2606" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2606" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2606" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2607">
+      <c r="A2607" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2607" t="n">
+        <v/>
+      </c>
+      <c r="C2607" t="inlineStr">
+        <is>
+          <t>https://www.spar.nl/vis-marine-kabeljauwfilets-4-stuks-9228133/</t>
+        </is>
+      </c>
+      <c r="D2607" t="inlineStr">
+        <is>
+          <t>Vis Marine Kabeljauw 400g</t>
+        </is>
+      </c>
+      <c r="E2607" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F2607" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="G2607" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2607" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2607" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2608">
+      <c r="A2608" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2608" t="n">
+        <v>27700</v>
+      </c>
+      <c r="C2608" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/309633</t>
+        </is>
+      </c>
+      <c r="D2608" t="inlineStr">
+        <is>
+          <t>528 ICE CUBES 1KG</t>
+        </is>
+      </c>
+      <c r="E2608" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2608" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2608" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2608" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2608" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2609">
+      <c r="A2609" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2609" t="n">
+        <v/>
+      </c>
+      <c r="C2609" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/vis-marine-koolvisfilets-doos-400-g-834796</t>
+        </is>
+      </c>
+      <c r="D2609" t="inlineStr">
+        <is>
+          <t>Vis Marine Koolvis 400g</t>
+        </is>
+      </c>
+      <c r="E2609" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F2609" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2609" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2609" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2609" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2610">
+      <c r="A2610" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2610" t="n">
+        <v/>
+      </c>
+      <c r="C2610" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/vis%20marine%20wilde%20zalm/96927</t>
+        </is>
+      </c>
+      <c r="D2610" t="inlineStr">
+        <is>
+          <t>Vis Marine Wilde zalm 540g</t>
+        </is>
+      </c>
+      <c r="E2610" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="F2610" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2610" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2610" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2610" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2611">
+      <c r="A2611" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2611" t="n">
+        <v/>
+      </c>
+      <c r="C2611" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/vis%20marine%20pangasiusfilet/82503</t>
+        </is>
+      </c>
+      <c r="D2611" t="inlineStr">
+        <is>
+          <t>Vis Marine Pangasiusfilet 540g</t>
+        </is>
+      </c>
+      <c r="E2611" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="F2611" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2611" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2611" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2611" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2612">
+      <c r="A2612" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2612" t="n">
+        <v/>
+      </c>
+      <c r="C2612" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/vis%20marine%20kabeljauwfilet%204%20stuks/49672</t>
+        </is>
+      </c>
+      <c r="D2612" t="inlineStr">
+        <is>
+          <t>Vis Marine Kabeljauw 400g</t>
+        </is>
+      </c>
+      <c r="E2612" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="F2612" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2612" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2612" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2612" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2613">
+      <c r="A2613" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2613" t="n">
+        <v/>
+      </c>
+      <c r="C2613" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/vis%20marine%20koolvisfilet%204%20stuks/49562</t>
+        </is>
+      </c>
+      <c r="D2613" t="inlineStr">
+        <is>
+          <t>Vis Marine Koolvis 400g</t>
+        </is>
+      </c>
+      <c r="E2613" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F2613" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2613" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2613" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2613" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2614">
+      <c r="A2614" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2614" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2614" t="inlineStr">
+        <is>
+          <t>https://www.spar.nl/queens-pangalicious-9158971/</t>
+        </is>
+      </c>
+      <c r="D2614" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2614" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="F2614" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="G2614" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2614" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2614" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2615">
+      <c r="A2615" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2615" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C2615" t="inlineStr">
+        <is>
+          <t>https://www.spar.nl/queens-pangasius-filet-citroen-peterselie-2730456/</t>
+        </is>
+      </c>
+      <c r="D2615" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS CITROEN &amp; PETERSELIE</t>
+        </is>
+      </c>
+      <c r="E2615" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="F2615" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="G2615" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2615" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2615" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2616">
+      <c r="A2616" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2616" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2616" t="inlineStr">
+        <is>
+          <t>https://www.spar.nl/queens-pangafilet-knoflook-kruiden-1998285/</t>
+        </is>
+      </c>
+      <c r="D2616" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2616" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="F2616" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="G2616" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2616" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2616" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2617">
+      <c r="A2617" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2617" t="n">
+        <v>27200</v>
+      </c>
+      <c r="C2617" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307851</t>
+        </is>
+      </c>
+      <c r="D2617" t="inlineStr">
+        <is>
+          <t>ORIEN BITES VEG GYOZA</t>
+        </is>
+      </c>
+      <c r="E2617" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="F2617" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2617" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2617" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2617" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2618">
+      <c r="A2618" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2618" t="n">
+        <v/>
+      </c>
+      <c r="C2618" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/vis-marine-kabeljauwfilets-msc-doos-540-g-723219</t>
+        </is>
+      </c>
+      <c r="D2618" t="inlineStr">
+        <is>
+          <t>Vis Marine Kabeljauw 540g</t>
+        </is>
+      </c>
+      <c r="E2618" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="F2618" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2618" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2618" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2618" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2619">
+      <c r="A2619" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2619" t="n">
+        <v>6541</v>
+      </c>
+      <c r="C2619" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20pangasiusfilet%20pikant%20gekruid/87324</t>
+        </is>
+      </c>
+      <c r="D2619" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS PIKANT GEKRUID</t>
+        </is>
+      </c>
+      <c r="E2619" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F2619" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2619" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2619" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2619" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2620">
+      <c r="A2620" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2620" t="n">
+        <v/>
+      </c>
+      <c r="C2620" t="inlineStr">
+        <is>
+          <t>https://www.aldi.nl/product/wilde-zalmfilets-1204877.html</t>
+        </is>
+      </c>
+      <c r="D2620" t="inlineStr">
+        <is>
+          <t>Aldi Wilde zalmfilet 500g</t>
+        </is>
+      </c>
+      <c r="E2620" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="F2620" t="inlineStr">
+        <is>
+          <t>Aldi</t>
+        </is>
+      </c>
+      <c r="G2620" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2620" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2620" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2621">
+      <c r="A2621" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2621" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C2621" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307713</t>
+        </is>
+      </c>
+      <c r="D2621" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS VISKROKANTJES NATUREL</t>
+        </is>
+      </c>
+      <c r="E2621" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F2621" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2621" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2621" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2621" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2622">
+      <c r="A2622" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2622" t="n">
+        <v/>
+      </c>
+      <c r="C2622" t="inlineStr">
+        <is>
+          <t>https://www.aldi.nl/product/pangasiusfilet-1221684.html</t>
+        </is>
+      </c>
+      <c r="D2622" t="inlineStr">
+        <is>
+          <t>Aldi Pangasiusfilet 540g</t>
+        </is>
+      </c>
+      <c r="E2622" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="F2622" t="inlineStr">
+        <is>
+          <t>Aldi</t>
+        </is>
+      </c>
+      <c r="G2622" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2622" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2622" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2623">
+      <c r="A2623" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2623" t="n">
+        <v/>
+      </c>
+      <c r="C2623" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi396815/ah-tilapiafilet-graatvrij</t>
+        </is>
+      </c>
+      <c r="D2623" t="inlineStr">
+        <is>
+          <t>AH Tilapiafilet graatvrij 225g</t>
+        </is>
+      </c>
+      <c r="E2623" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F2623" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2623" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2623" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2623" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2624">
+      <c r="A2624" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2624" t="n">
+        <v/>
+      </c>
+      <c r="C2624" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi178129/ah-wilde-zalmfilet</t>
+        </is>
+      </c>
+      <c r="D2624" t="inlineStr">
+        <is>
+          <t>AH Wilde zalmfilet 250g</t>
+        </is>
+      </c>
+      <c r="E2624" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="F2624" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2624" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2624" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2624" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2625">
+      <c r="A2625" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2625" t="n">
+        <v/>
+      </c>
+      <c r="C2625" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi141565/ah-wilde-zalmfilets</t>
+        </is>
+      </c>
+      <c r="D2625" t="inlineStr">
+        <is>
+          <t>AH Wilde zalmfilet 675g</t>
+        </is>
+      </c>
+      <c r="E2625" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="F2625" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2625" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2625" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2625" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2626">
+      <c r="A2626" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2626" t="n">
+        <v/>
+      </c>
+      <c r="C2626" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi140671/ah-pangasiusfilet</t>
+        </is>
+      </c>
+      <c r="D2626" t="inlineStr">
+        <is>
+          <t>AH Pangasiusfilet 675g</t>
+        </is>
+      </c>
+      <c r="E2626" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="F2626" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2626" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2626" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2626" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2627">
+      <c r="A2627" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2627" t="n">
+        <v/>
+      </c>
+      <c r="C2627" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi792/ah-kabeljauw</t>
+        </is>
+      </c>
+      <c r="D2627" t="inlineStr">
+        <is>
+          <t>AH Kabeljauw 400g</t>
+        </is>
+      </c>
+      <c r="E2627" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="F2627" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2627" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2627" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2627" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2628">
+      <c r="A2628" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2628" t="n">
+        <v/>
+      </c>
+      <c r="C2628" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi121478/ah-kabeljauwfilet</t>
+        </is>
+      </c>
+      <c r="D2628" t="inlineStr">
+        <is>
+          <t>AH Kabeljauwfilet 675g</t>
+        </is>
+      </c>
+      <c r="E2628" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="F2628" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2628" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2628" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2628" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2629">
+      <c r="A2629" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2629" t="n">
+        <v/>
+      </c>
+      <c r="C2629" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi39826/ah-koolvisfilet</t>
+        </is>
+      </c>
+      <c r="D2629" t="inlineStr">
+        <is>
+          <t>AH Koolvisfilet 400g</t>
+        </is>
+      </c>
+      <c r="E2629" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="F2629" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2629" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2629" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2629" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2630">
+      <c r="A2630" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2630" t="n">
+        <v/>
+      </c>
+      <c r="C2630" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-wilde-zalmfilet-2-x-125-g-76159PAK</t>
+        </is>
+      </c>
+      <c r="D2630" t="inlineStr">
+        <is>
+          <t>Jumbo Wilde Zalmfilet 2 x 125g</t>
+        </is>
+      </c>
+      <c r="E2630" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="F2630" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2630" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2630" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2630" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2631">
+      <c r="A2631" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2631" t="n">
+        <v/>
+      </c>
+      <c r="C2631" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/vismarine-koolvisfilet-4stmsc/811408</t>
+        </is>
+      </c>
+      <c r="D2631" t="inlineStr">
+        <is>
+          <t>Vis Marine Koolvis 400g</t>
+        </is>
+      </c>
+      <c r="E2631" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F2631" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2631" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2631" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2631" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2632">
+      <c r="A2632" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2632" t="n">
+        <v>27207</v>
+      </c>
+      <c r="C2632" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307850</t>
+        </is>
+      </c>
+      <c r="D2632" t="inlineStr">
+        <is>
+          <t>ORIEN BITES CHICKEN GYOZA</t>
+        </is>
+      </c>
+      <c r="E2632" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="F2632" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2632" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2632" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2632" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2633">
+      <c r="A2633" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2633" t="n">
+        <v/>
+      </c>
+      <c r="C2633" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-pangasiusfilet-270-g-173837ZK</t>
+        </is>
+      </c>
+      <c r="D2633" t="inlineStr">
+        <is>
+          <t>Jumbo Pangasiusfilet 270g</t>
+        </is>
+      </c>
+      <c r="E2633" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="F2633" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2633" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2633" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2633" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2634">
+      <c r="A2634" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2634" t="n">
+        <v/>
+      </c>
+      <c r="C2634" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-pangasiusfilet-vriesvers-675-g-494433ZK</t>
+        </is>
+      </c>
+      <c r="D2634" t="inlineStr">
+        <is>
+          <t>Jumbo Pangasiusfilet Vriesvers 675g</t>
+        </is>
+      </c>
+      <c r="E2634" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F2634" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2634" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2634" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2634" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2635">
+      <c r="A2635" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2635" t="n">
+        <v/>
+      </c>
+      <c r="C2635" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-kabeljauwfilet-675-g-471158ZK</t>
+        </is>
+      </c>
+      <c r="D2635" t="inlineStr">
+        <is>
+          <t>Jumbo Kabeljauwfilet 675g</t>
+        </is>
+      </c>
+      <c r="E2635" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="F2635" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2635" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2635" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2635" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2636">
+      <c r="A2636" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2636" t="n">
+        <v/>
+      </c>
+      <c r="C2636" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/seacon-alaska-koolvisfilet-675g-706749ZK</t>
+        </is>
+      </c>
+      <c r="D2636" t="inlineStr">
+        <is>
+          <t>Seacon Alaska Koolvisfilet 675g</t>
+        </is>
+      </c>
+      <c r="E2636" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="F2636" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2636" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2636" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2636" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2637">
+      <c r="A2637" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2637" t="n">
+        <v/>
+      </c>
+      <c r="C2637" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-koolvis-filet-400-g-713748DS</t>
+        </is>
+      </c>
+      <c r="D2637" t="inlineStr">
+        <is>
+          <t>Jumbo Koolvis Filet 400g</t>
+        </is>
+      </c>
+      <c r="E2637" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F2637" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2637" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2637" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2637" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2638">
+      <c r="A2638" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2638" t="n">
+        <v/>
+      </c>
+      <c r="C2638" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis-marine-tilapia-filets-5-6-st/83124</t>
+        </is>
+      </c>
+      <c r="D2638" t="inlineStr">
+        <is>
+          <t>Vis Marine Tilapiafilets 540g</t>
+        </is>
+      </c>
+      <c r="E2638" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="F2638" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2638" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2638" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2638" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2639">
+      <c r="A2639" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2639" t="n">
+        <v/>
+      </c>
+      <c r="C2639" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis%20marine%20wilde%20zalm/96927</t>
+        </is>
+      </c>
+      <c r="D2639" t="inlineStr">
+        <is>
+          <t>Vis Marine Wilde zalm 540g</t>
+        </is>
+      </c>
+      <c r="E2639" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="F2639" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2639" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2639" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2639" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2640">
+      <c r="A2640" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2640" t="n">
+        <v/>
+      </c>
+      <c r="C2640" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis%20marine%20pangasiusfilet/82503</t>
+        </is>
+      </c>
+      <c r="D2640" t="inlineStr">
+        <is>
+          <t>Vis Marine Pangasiusfilet 540g</t>
+        </is>
+      </c>
+      <c r="E2640" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="F2640" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2640" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2640" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2640" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2641">
+      <c r="A2641" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2641" t="n">
+        <v/>
+      </c>
+      <c r="C2641" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis%20marine%20kabeljauwfilets/111544</t>
+        </is>
+      </c>
+      <c r="D2641" t="inlineStr">
+        <is>
+          <t>Vis Marine Kabeljauw 540g</t>
+        </is>
+      </c>
+      <c r="F2641" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2641" t="inlineStr">
+        <is>
+          <t>Niet beschikbaar</t>
+        </is>
+      </c>
+      <c r="H2641" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2641" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2642">
+      <c r="A2642" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2642" t="n">
+        <v/>
+      </c>
+      <c r="C2642" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/vis%20marine%20koolvisfilet%204%20stuks/49562</t>
+        </is>
+      </c>
+      <c r="D2642" t="inlineStr">
+        <is>
+          <t>Vis Marine Koolvis 400g</t>
+        </is>
+      </c>
+      <c r="E2642" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F2642" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2642" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2642" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2642" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2643">
+      <c r="A2643" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2643" t="n">
+        <v/>
+      </c>
+      <c r="C2643" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/jumbo-zalmfilet-met-huid-2-x-125-g-723226DS</t>
+        </is>
+      </c>
+      <c r="D2643" t="inlineStr">
+        <is>
+          <t>Jumbo Zalmfilet met Huid 2 x 125g</t>
+        </is>
+      </c>
+      <c r="E2643" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="F2643" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2643" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2643" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2643" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2644">
+      <c r="A2644" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2644" t="n">
+        <v/>
+      </c>
+      <c r="C2644" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/vismarine-pangasiusfilet-540gr/110960</t>
+        </is>
+      </c>
+      <c r="D2644" t="inlineStr">
+        <is>
+          <t>Vis Marine Pangasiusfilet 540g</t>
+        </is>
+      </c>
+      <c r="E2644" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="F2644" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2644" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2644" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2644" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2645">
+      <c r="A2645" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2645" t="n">
+        <v/>
+      </c>
+      <c r="C2645" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/vis-marine-kabeljauwfilets</t>
+        </is>
+      </c>
+      <c r="D2645" t="inlineStr">
+        <is>
+          <t>Vis Marine Kabeljauw 400g</t>
+        </is>
+      </c>
+      <c r="E2645" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="F2645" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2645" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2645" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2645" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2646">
+      <c r="A2646" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2646" t="n">
+        <v>6989</v>
+      </c>
+      <c r="C2646" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi212118/ah-ijsblokjes</t>
+        </is>
+      </c>
+      <c r="D2646" t="inlineStr">
+        <is>
+          <t>ALBERT HEIJN IJSBLOKJES 1KG</t>
+        </is>
+      </c>
+      <c r="E2646" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F2646" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2646" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2646" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2646" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2647">
+      <c r="A2647" t="inlineStr">
+        <is>
+          <t>Concurrent</t>
+        </is>
+      </c>
+      <c r="B2647" t="n">
+        <v/>
+      </c>
+      <c r="C2647" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/vis-marine-wilde-zalm</t>
+        </is>
+      </c>
+      <c r="D2647" t="inlineStr">
+        <is>
+          <t>Vis Marine Wilde zalm 540g</t>
+        </is>
+      </c>
+      <c r="E2647" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="F2647" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2647" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2647" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2647" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2648">
+      <c r="A2648" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2648" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2648" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307674</t>
+        </is>
+      </c>
+      <c r="D2648" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2648" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F2648" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2648" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2648" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2648" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2649">
+      <c r="A2649" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2649" t="n">
+        <v>27703</v>
+      </c>
+      <c r="C2649" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/528-crushed-ice-zak-2-kg-318163</t>
+        </is>
+      </c>
+      <c r="D2649" t="inlineStr">
+        <is>
+          <t>528 CRUSHED ICE 2KG</t>
+        </is>
+      </c>
+      <c r="E2649" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="F2649" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2649" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2649" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2649" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2650">
+      <c r="A2650" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2650" t="n">
+        <v>27701</v>
+      </c>
+      <c r="C2650" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/528-ijsblokjes-zak-2-kg-243144</t>
+        </is>
+      </c>
+      <c r="D2650" t="inlineStr">
+        <is>
+          <t>528 ICE CUBES 2KG</t>
+        </is>
+      </c>
+      <c r="E2650" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="F2650" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2650" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2650" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2650" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2651">
+      <c r="A2651" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2651" t="n">
+        <v>15594</v>
+      </c>
+      <c r="C2651" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/neutraal-knoflookbaguette-zak-175-g-455342</t>
+        </is>
+      </c>
+      <c r="D2651" t="inlineStr">
+        <is>
+          <t>KNOFLOOKBAGUETTE</t>
+        </is>
+      </c>
+      <c r="E2651" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F2651" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2651" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2651" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2651" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2652">
+      <c r="A2652" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2652" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2652" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/queens-pangalicious-extra-krokant-doos-250-g-439896</t>
+        </is>
+      </c>
+      <c r="D2652" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2652" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F2652" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2652" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2652" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2652" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2653">
+      <c r="A2653" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2653" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C2653" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/queens-pangalicious-citroen-peterselie-doos-250-g-811995</t>
+        </is>
+      </c>
+      <c r="D2653" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS CITROEN &amp; PETERSELIE</t>
+        </is>
+      </c>
+      <c r="E2653" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2653" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2653" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2653" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2653" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2654">
+      <c r="A2654" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2654" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2654" t="inlineStr">
+        <is>
+          <t>https://www.plus.nl/product/queens-pangalicious-knoflook-kruiden-doos-250-g-439900</t>
+        </is>
+      </c>
+      <c r="D2654" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2654" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2654" t="inlineStr">
+        <is>
+          <t>Plus</t>
+        </is>
+      </c>
+      <c r="G2654" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2654" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2654" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2655">
+      <c r="A2655" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2655" t="n">
+        <v>6097</v>
+      </c>
+      <c r="C2655" t="inlineStr">
+        <is>
+          <t>https://www.aldi.nl/product-detail/gepaneerde-pangasiusfilets-1219976.html</t>
+        </is>
+      </c>
+      <c r="D2655" t="inlineStr">
+        <is>
+          <t>GOLDEN SEAFOOD ASC GEPANEERDE PANGASIUSFILET 6097</t>
+        </is>
+      </c>
+      <c r="E2655" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F2655" t="inlineStr">
+        <is>
+          <t>Aldi</t>
+        </is>
+      </c>
+      <c r="G2655" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2655" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2655" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2656">
+      <c r="A2656" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2656" t="n">
+        <v>27208</v>
+      </c>
+      <c r="C2656" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/orienbites-gua-bao-320g-702769DS</t>
+        </is>
+      </c>
+      <c r="D2656" t="inlineStr">
+        <is>
+          <t>ORIEN BITES GUA BAO 320g</t>
+        </is>
+      </c>
+      <c r="E2656" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F2656" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2656" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2656" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2656" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2657">
+      <c r="A2657" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2657" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C2657" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-pangalicious-krokantjes-naturel-pangasiusfilet-250-g-doos-697050DS</t>
+        </is>
+      </c>
+      <c r="D2657" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS VISKROKANTJES NATUREL</t>
+        </is>
+      </c>
+      <c r="E2657" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2657" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2657" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2657" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2657" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2658">
+      <c r="A2658" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2658" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2658" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/queens-panga-extra-krokant/148518</t>
+        </is>
+      </c>
+      <c r="D2658" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2658" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F2658" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2658" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2658" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2658" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2659">
+      <c r="A2659" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2659" t="n">
+        <v>5960</v>
+      </c>
+      <c r="C2659" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/queens-pangafilets2</t>
+        </is>
+      </c>
+      <c r="D2659" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGAFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2659" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F2659" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2659" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2659" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2659" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2660">
+      <c r="A2660" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2660" t="n">
+        <v>5960</v>
+      </c>
+      <c r="C2660" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-panga-filets-375-g-419420ZK</t>
+        </is>
+      </c>
+      <c r="D2660" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGAFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2660" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F2660" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2660" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2660" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2660" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2661">
+      <c r="A2661" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2661" t="n">
+        <v>5960</v>
+      </c>
+      <c r="C2661" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20pangafilet/42053</t>
+        </is>
+      </c>
+      <c r="D2661" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGAFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2661" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F2661" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2661" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2661" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2661" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2662">
+      <c r="A2662" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2662" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C2662" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307667</t>
+        </is>
+      </c>
+      <c r="D2662" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS CITROEN &amp; PETERSELIE</t>
+        </is>
+      </c>
+      <c r="E2662" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F2662" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2662" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2662" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2662" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2663">
+      <c r="A2663" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2663" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2663" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20pangalicious%20knoflook%20kruiden/30297</t>
+        </is>
+      </c>
+      <c r="D2663" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2663" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="F2663" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2663" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2663" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2663" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2664">
+      <c r="A2664" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2664" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2664" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20pangalicious%20extra%20krokant/35468</t>
+        </is>
+      </c>
+      <c r="D2664" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2664" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F2664" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2664" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2664" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2664" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2665">
+      <c r="A2665" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2665" t="n">
+        <v>27702</v>
+      </c>
+      <c r="C2665" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/the-ice-co-scherfijs</t>
+        </is>
+      </c>
+      <c r="D2665" t="inlineStr">
+        <is>
+          <t>528 CRUSHED ICE 1KG</t>
+        </is>
+      </c>
+      <c r="E2665" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="F2665" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2665" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2665" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2665" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2666">
+      <c r="A2666" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2666" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C2666" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/queens-pangalicious-citroen-peterselie1</t>
+        </is>
+      </c>
+      <c r="D2666" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS CITROEN &amp; PETERSELIE</t>
+        </is>
+      </c>
+      <c r="E2666" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="F2666" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2666" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2666" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2666" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2667">
+      <c r="A2667" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2667" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2667" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/queens-pangalicious-ex-krokant</t>
+        </is>
+      </c>
+      <c r="D2667" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2667" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F2667" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2667" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2667" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2667" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2668">
+      <c r="A2668" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2668" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2668" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/queens-pangalicious-knoflook-kruiden1</t>
+        </is>
+      </c>
+      <c r="D2668" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2668" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="F2668" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2668" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2668" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2668" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2669">
+      <c r="A2669" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2669" t="n">
+        <v>5962</v>
+      </c>
+      <c r="C2669" t="inlineStr">
+        <is>
+          <t>https://www.hoogvliet.com/product/queens-wilde-zalmfilet-met-huid</t>
+        </is>
+      </c>
+      <c r="D2669" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ZALMFILET MET HUID 375G</t>
+        </is>
+      </c>
+      <c r="E2669" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="F2669" t="inlineStr">
+        <is>
+          <t>Hoogvliet</t>
+        </is>
+      </c>
+      <c r="G2669" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2669" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2669" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2670">
+      <c r="A2670" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2670" t="n">
+        <v>7001</v>
+      </c>
+      <c r="C2670" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-pangalicious-krokantjes-gekruid-pangasiusfilet-250g-697039DS</t>
+        </is>
+      </c>
+      <c r="D2670" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS VISKROKANTJES GEKRUID</t>
+        </is>
+      </c>
+      <c r="E2670" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2670" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2670" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2670" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2670" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2671">
+      <c r="A2671" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2671" t="n">
+        <v>27704</v>
+      </c>
+      <c r="C2671" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/528-ijsballen-1-kg-741532ZK</t>
+        </is>
+      </c>
+      <c r="D2671" t="inlineStr">
+        <is>
+          <t>528 ICE BALLS 1KG</t>
+        </is>
+      </c>
+      <c r="E2671" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="F2671" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2671" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2671" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2671" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2672">
+      <c r="A2672" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2672" t="n">
+        <v>5961</v>
+      </c>
+      <c r="C2672" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-alaska-koolvis-filets-375-g-419422ZK</t>
+        </is>
+      </c>
+      <c r="D2672" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ALASKA KOOLVISFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2672" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="F2672" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2672" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2672" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2672" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2673">
+      <c r="A2673" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2673" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2673" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-pangalicious-extra-krokant-2-stuks-250-g-184995DS</t>
+        </is>
+      </c>
+      <c r="D2673" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2673" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F2673" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2673" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2673" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2673" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2674">
+      <c r="A2674" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2674" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2674" t="inlineStr">
+        <is>
+          <t>https://webwinkel.poiesz-supermarkten.nl/boodschappen/producten/307666</t>
+        </is>
+      </c>
+      <c r="D2674" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2674" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F2674" t="inlineStr">
+        <is>
+          <t>Poiesz</t>
+        </is>
+      </c>
+      <c r="G2674" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2674" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2674" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2675">
+      <c r="A2675" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2675" t="n">
+        <v>5960</v>
+      </c>
+      <c r="C2675" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20pangafilet/42053</t>
+        </is>
+      </c>
+      <c r="D2675" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGAFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2675" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="F2675" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2675" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2675" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2675" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2676">
+      <c r="A2676" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2676" t="n">
+        <v>5961</v>
+      </c>
+      <c r="C2676" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/queens-koolvis-375gr/137392</t>
+        </is>
+      </c>
+      <c r="D2676" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ALASKA KOOLVISFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2676" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2676" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2676" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2676" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2676" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2677">
+      <c r="A2677" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2677" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2677" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/queens-panga-knof-kruid-250gr/125556</t>
+        </is>
+      </c>
+      <c r="D2677" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2677" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="F2677" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2677" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2677" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2677" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2678">
+      <c r="A2678" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2678" t="n">
+        <v>6673</v>
+      </c>
+      <c r="C2678" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20kabeljauwfilet%20met%20huid/115384</t>
+        </is>
+      </c>
+      <c r="D2678" t="inlineStr">
+        <is>
+          <t>QUEENS MSC KABELJAUWFILETS MET HUID 375G</t>
+        </is>
+      </c>
+      <c r="E2678" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="F2678" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2678" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2678" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2678" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2679">
+      <c r="A2679" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2679" t="n">
+        <v>5960</v>
+      </c>
+      <c r="C2679" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/queens-pangafilets-375gr/134358</t>
+        </is>
+      </c>
+      <c r="D2679" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGAFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2679" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F2679" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2679" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2679" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2679" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2680">
+      <c r="A2680" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2680" t="n">
+        <v>6541</v>
+      </c>
+      <c r="C2680" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20pangasiusfilet%20pikant%20gekruid/87324</t>
+        </is>
+      </c>
+      <c r="D2680" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS PIKANT GEKRUID</t>
+        </is>
+      </c>
+      <c r="E2680" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="F2680" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2680" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2680" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2680" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2681">
+      <c r="A2681" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2681" t="n">
+        <v>6534</v>
+      </c>
+      <c r="C2681" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20pangalicious%20extra%20krokant/35468</t>
+        </is>
+      </c>
+      <c r="D2681" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS EXTRA KROKANT</t>
+        </is>
+      </c>
+      <c r="E2681" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F2681" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2681" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2681" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2681" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2682">
+      <c r="A2682" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2682" t="n">
+        <v>5962</v>
+      </c>
+      <c r="C2682" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20wilde%20zalmfilets%20met%20huid/59292</t>
+        </is>
+      </c>
+      <c r="D2682" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ZALMFILET MET HUID 375G</t>
+        </is>
+      </c>
+      <c r="E2682" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="F2682" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2682" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2682" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2682" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2683">
+      <c r="A2683" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2683" t="n">
+        <v>5961</v>
+      </c>
+      <c r="C2683" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20alaska%20koolvisfilet/42054</t>
+        </is>
+      </c>
+      <c r="D2683" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ALASKA KOOLVISFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2683" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="F2683" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2683" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2683" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2683" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2684">
+      <c r="A2684" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2684" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2684" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20pangalicious%20knoflook%20kruiden/30297</t>
+        </is>
+      </c>
+      <c r="D2684" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2684" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F2684" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2684" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2684" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2684" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2685">
+      <c r="A2685" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2685" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C2685" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20pangalicious%20citroen-peterselie/32212</t>
+        </is>
+      </c>
+      <c r="D2685" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS CITROEN &amp; PETERSELIE</t>
+        </is>
+      </c>
+      <c r="E2685" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="F2685" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2685" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2685" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2685" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2686">
+      <c r="A2686" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2686" t="n">
+        <v>27702</v>
+      </c>
+      <c r="C2686" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/ijs/crushed%20ijs/116221</t>
+        </is>
+      </c>
+      <c r="D2686" t="inlineStr">
+        <is>
+          <t>528 CRUSHED ICE 1KG</t>
+        </is>
+      </c>
+      <c r="F2686" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2686" t="inlineStr">
+        <is>
+          <t>Geen prijs gevonden</t>
+        </is>
+      </c>
+      <c r="H2686" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2686" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2687">
+      <c r="A2687" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2687" t="n">
+        <v>5962</v>
+      </c>
+      <c r="C2687" t="inlineStr">
+        <is>
+          <t>https://www.vomar.nl/producten/diepvries/diepvries-vis-schaaldieren/queens-wilde-zalmfilet/154077</t>
+        </is>
+      </c>
+      <c r="D2687" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ZALMFILET MET HUID 375G</t>
+        </is>
+      </c>
+      <c r="E2687" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="F2687" t="inlineStr">
+        <is>
+          <t>Vomar</t>
+        </is>
+      </c>
+      <c r="G2687" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2687" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2687" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2688">
+      <c r="A2688" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2688" t="n">
+        <v>15594</v>
+      </c>
+      <c r="C2688" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-snacks/queens%20baguette%20met%20knoflookboter/118061</t>
+        </is>
+      </c>
+      <c r="D2688" t="inlineStr">
+        <is>
+          <t>KNOFLOOKBAGUETTE</t>
+        </is>
+      </c>
+      <c r="F2688" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2688" t="inlineStr">
+        <is>
+          <t>Geen prijs gevonden</t>
+        </is>
+      </c>
+      <c r="H2688" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2688" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2689">
+      <c r="A2689" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2689" t="n">
+        <v>5961</v>
+      </c>
+      <c r="C2689" t="inlineStr">
+        <is>
+          <t>https://www.dirk.nl/boodschappen/diepvries/diepvries-vis/queens%20alaska%20koolvisfilet/42054</t>
+        </is>
+      </c>
+      <c r="D2689" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ALASKA KOOLVISFILET 375G</t>
+        </is>
+      </c>
+      <c r="E2689" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2689" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="G2689" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2689" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2689" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2690">
+      <c r="A2690" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2690" t="n">
+        <v>27702</v>
+      </c>
+      <c r="C2690" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/ijs/crushed%20ijs/116221</t>
+        </is>
+      </c>
+      <c r="D2690" t="inlineStr">
+        <is>
+          <t>528 CRUSHED ICE 1KG</t>
+        </is>
+      </c>
+      <c r="E2690" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F2690" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2690" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2690" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2690" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2691">
+      <c r="A2691" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2691" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C2691" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-pangalicious-citroen-peterselie-2-stuks-250-g-184997DS</t>
+        </is>
+      </c>
+      <c r="D2691" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS CITROEN &amp; PETERSELIE</t>
+        </is>
+      </c>
+      <c r="E2691" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2691" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2691" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2691" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2691" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2692">
+      <c r="A2692" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2692" t="n">
+        <v>6673</v>
+      </c>
+      <c r="C2692" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-kabeljauwfilet-met-huid-375g-705923ZK</t>
+        </is>
+      </c>
+      <c r="D2692" t="inlineStr">
+        <is>
+          <t>QUEENS MSC KABELJAUWFILETS MET HUID 375G</t>
+        </is>
+      </c>
+      <c r="F2692" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2692" t="inlineStr">
+        <is>
+          <t>Geen prijs gevonden</t>
+        </is>
+      </c>
+      <c r="H2692" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2692" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2693">
+      <c r="A2693" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2693" t="n">
+        <v>6541</v>
+      </c>
+      <c r="C2693" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-pangalicious-pikant-gekruid-2-stuks-250-g-550475DS</t>
+        </is>
+      </c>
+      <c r="D2693" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS PIKANT GEKRUID</t>
+        </is>
+      </c>
+      <c r="E2693" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="F2693" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2693" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2693" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2693" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2694">
+      <c r="A2694" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2694" t="n">
+        <v>27704</v>
+      </c>
+      <c r="C2694" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi589548/528-premium-ice-balls</t>
+        </is>
+      </c>
+      <c r="D2694" t="inlineStr">
+        <is>
+          <t>528 ICE BALLS 1KG</t>
+        </is>
+      </c>
+      <c r="F2694" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2694" t="inlineStr">
+        <is>
+          <t>Geen prijs gevonden</t>
+        </is>
+      </c>
+      <c r="H2694" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2694" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2695">
+      <c r="A2695" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2695" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C2695" t="inlineStr">
+        <is>
+          <t>https://www.jumbo.com/producten/queens-pangalicious-knoflook-kruiden-2-stuks-250-g-184996DS</t>
+        </is>
+      </c>
+      <c r="D2695" t="inlineStr">
+        <is>
+          <t>QUEENS ASC PANGALICIOUS KNOFLOOK &amp; KRUIDEN</t>
+        </is>
+      </c>
+      <c r="E2695" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F2695" t="inlineStr">
+        <is>
+          <t>Jumbo</t>
+        </is>
+      </c>
+      <c r="G2695" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2695" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2695" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2696">
+      <c r="A2696" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2696" t="n">
+        <v>5962</v>
+      </c>
+      <c r="C2696" t="inlineStr">
+        <is>
+          <t>https://www.dekamarkt.nl/producten/diepvries/diepvries-vis/queens%20wilde%20zalmfilets%20met%20huid/59292</t>
+        </is>
+      </c>
+      <c r="D2696" t="inlineStr">
+        <is>
+          <t>QUEENS MSC ZALMFILET MET HUID 375G</t>
+        </is>
+      </c>
+      <c r="E2696" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="F2696" t="inlineStr">
+        <is>
+          <t>DekaMarkt</t>
+        </is>
+      </c>
+      <c r="G2696" t="inlineStr">
+        <is>
+          <t>Succes (Visueel HTML)</t>
+        </is>
+      </c>
+      <c r="H2696" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2696" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2697">
+      <c r="A2697" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2697" t="n">
+        <v>17025</v>
+      </c>
+      <c r="C2697" t="inlineStr">
+        <is>
+          <t>https://www.ah.nl/producten/product/wi599401/ah-ijs-spinners</t>
+        </is>
+      </c>
+      <c r="D2697" t="inlineStr">
+        <is>
+          <t>AH SPINNER AARDBEI SINAASAPPEL VANILLE</t>
+        </is>
+      </c>
+      <c r="E2697" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="F2697" t="inlineStr">
+        <is>
+          <t>Albert Heijn</t>
+        </is>
+      </c>
+      <c r="G2697" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2697" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2697" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="2698">
+      <c r="A2698" t="inlineStr">
+        <is>
+          <t>Queens</t>
+        </is>
+      </c>
+      <c r="B2698" t="n">
+        <v>17300</v>
+      </c>
+      <c r="C2698" t="inlineStr">
+        <is>
+          <t>https://www.aldi.nl/product/spinner-ijs-1232061.html</t>
+        </is>
+      </c>
+      <c r="D2698" t="inlineStr">
+        <is>
+          <t>MUCCI SPINNER AARDBEI VANILLE</t>
+        </is>
+      </c>
+      <c r="E2698" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="F2698" t="inlineStr">
+        <is>
+          <t>Aldi</t>
+        </is>
+      </c>
+      <c r="G2698" t="inlineStr">
+        <is>
+          <t>Succes (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="H2698" s="13" t="n">
+        <v>46168</v>
+      </c>
+      <c r="I2698" t="n">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId1"/>

</xml_diff>